<commit_message>
ci: update android-e2e workflow with passing test suite & github pages publish
</commit_message>
<xml_diff>
--- a/automation/reports/Excel/Passed_Test_Cases.xlsx
+++ b/automation/reports/Excel/Passed_Test_Cases.xlsx
@@ -3591,7 +3591,7 @@
         <v>10</v>
       </c>
       <c r="F2">
-        <v>981</v>
+        <v>354</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -3611,7 +3611,7 @@
         <v>10</v>
       </c>
       <c r="F3">
-        <v>933</v>
+        <v>448</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -3631,7 +3631,7 @@
         <v>10</v>
       </c>
       <c r="F4">
-        <v>823</v>
+        <v>616</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -3651,7 +3651,7 @@
         <v>10</v>
       </c>
       <c r="F5">
-        <v>535</v>
+        <v>815</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -3671,7 +3671,7 @@
         <v>10</v>
       </c>
       <c r="F6">
-        <v>359</v>
+        <v>919</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -3691,7 +3691,7 @@
         <v>10</v>
       </c>
       <c r="F7">
-        <v>633</v>
+        <v>931</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -3711,7 +3711,7 @@
         <v>10</v>
       </c>
       <c r="F8">
-        <v>682</v>
+        <v>961</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -3731,7 +3731,7 @@
         <v>10</v>
       </c>
       <c r="F9">
-        <v>213</v>
+        <v>271</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -3751,7 +3751,7 @@
         <v>10</v>
       </c>
       <c r="F10">
-        <v>833</v>
+        <v>530</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -3771,7 +3771,7 @@
         <v>10</v>
       </c>
       <c r="F11">
-        <v>704</v>
+        <v>488</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -3791,7 +3791,7 @@
         <v>10</v>
       </c>
       <c r="F12">
-        <v>223</v>
+        <v>636</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
@@ -3811,7 +3811,7 @@
         <v>10</v>
       </c>
       <c r="F13">
-        <v>410</v>
+        <v>753</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
@@ -3831,7 +3831,7 @@
         <v>10</v>
       </c>
       <c r="F14">
-        <v>831</v>
+        <v>386</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
@@ -3851,7 +3851,7 @@
         <v>10</v>
       </c>
       <c r="F15">
-        <v>868</v>
+        <v>835</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
@@ -3871,7 +3871,7 @@
         <v>10</v>
       </c>
       <c r="F16">
-        <v>678</v>
+        <v>712</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
@@ -3891,7 +3891,7 @@
         <v>10</v>
       </c>
       <c r="F17">
-        <v>906</v>
+        <v>563</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
@@ -3911,7 +3911,7 @@
         <v>10</v>
       </c>
       <c r="F18">
-        <v>524</v>
+        <v>284</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
@@ -3931,7 +3931,7 @@
         <v>10</v>
       </c>
       <c r="F19">
-        <v>541</v>
+        <v>837</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
@@ -3951,7 +3951,7 @@
         <v>10</v>
       </c>
       <c r="F20">
-        <v>285</v>
+        <v>220</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
@@ -3971,7 +3971,7 @@
         <v>10</v>
       </c>
       <c r="F21">
-        <v>631</v>
+        <v>807</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
@@ -3991,7 +3991,7 @@
         <v>10</v>
       </c>
       <c r="F22">
-        <v>876</v>
+        <v>225</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
@@ -4011,7 +4011,7 @@
         <v>10</v>
       </c>
       <c r="F23">
-        <v>374</v>
+        <v>999</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
@@ -4031,7 +4031,7 @@
         <v>10</v>
       </c>
       <c r="F24">
-        <v>626</v>
+        <v>487</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
@@ -4051,7 +4051,7 @@
         <v>10</v>
       </c>
       <c r="F25">
-        <v>352</v>
+        <v>344</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
@@ -4071,7 +4071,7 @@
         <v>10</v>
       </c>
       <c r="F26">
-        <v>268</v>
+        <v>219</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
@@ -4091,7 +4091,7 @@
         <v>10</v>
       </c>
       <c r="F27">
-        <v>667</v>
+        <v>671</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
@@ -4111,7 +4111,7 @@
         <v>10</v>
       </c>
       <c r="F28">
-        <v>841</v>
+        <v>205</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
@@ -4131,7 +4131,7 @@
         <v>10</v>
       </c>
       <c r="F29">
-        <v>318</v>
+        <v>923</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
@@ -4151,7 +4151,7 @@
         <v>10</v>
       </c>
       <c r="F30">
-        <v>773</v>
+        <v>298</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
@@ -4171,7 +4171,7 @@
         <v>10</v>
       </c>
       <c r="F31">
-        <v>575</v>
+        <v>219</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
@@ -4191,7 +4191,7 @@
         <v>10</v>
       </c>
       <c r="F32">
-        <v>373</v>
+        <v>558</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
@@ -4211,7 +4211,7 @@
         <v>10</v>
       </c>
       <c r="F33">
-        <v>321</v>
+        <v>684</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
@@ -4231,7 +4231,7 @@
         <v>10</v>
       </c>
       <c r="F34">
-        <v>537</v>
+        <v>459</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
@@ -4251,7 +4251,7 @@
         <v>10</v>
       </c>
       <c r="F35">
-        <v>498</v>
+        <v>439</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
@@ -4271,7 +4271,7 @@
         <v>10</v>
       </c>
       <c r="F36">
-        <v>243</v>
+        <v>793</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
@@ -4291,7 +4291,7 @@
         <v>10</v>
       </c>
       <c r="F37">
-        <v>799</v>
+        <v>843</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
@@ -4311,7 +4311,7 @@
         <v>10</v>
       </c>
       <c r="F38">
-        <v>893</v>
+        <v>294</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
@@ -4331,7 +4331,7 @@
         <v>10</v>
       </c>
       <c r="F39">
-        <v>215</v>
+        <v>326</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
@@ -4351,7 +4351,7 @@
         <v>10</v>
       </c>
       <c r="F40">
-        <v>454</v>
+        <v>387</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
@@ -4371,7 +4371,7 @@
         <v>10</v>
       </c>
       <c r="F41">
-        <v>534</v>
+        <v>644</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
@@ -4391,7 +4391,7 @@
         <v>10</v>
       </c>
       <c r="F42">
-        <v>759</v>
+        <v>780</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -4411,7 +4411,7 @@
         <v>10</v>
       </c>
       <c r="F43">
-        <v>848</v>
+        <v>673</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
@@ -4431,7 +4431,7 @@
         <v>10</v>
       </c>
       <c r="F44">
-        <v>676</v>
+        <v>911</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -4451,7 +4451,7 @@
         <v>10</v>
       </c>
       <c r="F45">
-        <v>980</v>
+        <v>418</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -4471,7 +4471,7 @@
         <v>10</v>
       </c>
       <c r="F46">
-        <v>857</v>
+        <v>349</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
@@ -4491,7 +4491,7 @@
         <v>10</v>
       </c>
       <c r="F47">
-        <v>502</v>
+        <v>405</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -4511,7 +4511,7 @@
         <v>10</v>
       </c>
       <c r="F48">
-        <v>317</v>
+        <v>511</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -4531,7 +4531,7 @@
         <v>10</v>
       </c>
       <c r="F49">
-        <v>291</v>
+        <v>368</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
@@ -4551,7 +4551,7 @@
         <v>10</v>
       </c>
       <c r="F50">
-        <v>498</v>
+        <v>934</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
@@ -4571,7 +4571,7 @@
         <v>10</v>
       </c>
       <c r="F51">
-        <v>504</v>
+        <v>599</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
@@ -4591,7 +4591,7 @@
         <v>10</v>
       </c>
       <c r="F52">
-        <v>629</v>
+        <v>878</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
@@ -4611,7 +4611,7 @@
         <v>10</v>
       </c>
       <c r="F53">
-        <v>575</v>
+        <v>605</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
@@ -4631,7 +4631,7 @@
         <v>10</v>
       </c>
       <c r="F54">
-        <v>750</v>
+        <v>981</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
@@ -4651,7 +4651,7 @@
         <v>10</v>
       </c>
       <c r="F55">
-        <v>910</v>
+        <v>250</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
@@ -4671,7 +4671,7 @@
         <v>10</v>
       </c>
       <c r="F56">
-        <v>492</v>
+        <v>321</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
@@ -4691,7 +4691,7 @@
         <v>10</v>
       </c>
       <c r="F57">
-        <v>870</v>
+        <v>788</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
@@ -4711,7 +4711,7 @@
         <v>10</v>
       </c>
       <c r="F58">
-        <v>432</v>
+        <v>441</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
@@ -4731,7 +4731,7 @@
         <v>10</v>
       </c>
       <c r="F59">
-        <v>489</v>
+        <v>684</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
@@ -4751,7 +4751,7 @@
         <v>10</v>
       </c>
       <c r="F60">
-        <v>536</v>
+        <v>414</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
@@ -4771,7 +4771,7 @@
         <v>10</v>
       </c>
       <c r="F61">
-        <v>731</v>
+        <v>679</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
@@ -4791,7 +4791,7 @@
         <v>10</v>
       </c>
       <c r="F62">
-        <v>405</v>
+        <v>953</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
@@ -4811,7 +4811,7 @@
         <v>10</v>
       </c>
       <c r="F63">
-        <v>537</v>
+        <v>910</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
@@ -4831,7 +4831,7 @@
         <v>10</v>
       </c>
       <c r="F64">
-        <v>434</v>
+        <v>261</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
@@ -4851,7 +4851,7 @@
         <v>10</v>
       </c>
       <c r="F65">
-        <v>789</v>
+        <v>590</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
@@ -4871,7 +4871,7 @@
         <v>10</v>
       </c>
       <c r="F66">
-        <v>953</v>
+        <v>547</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
@@ -4891,7 +4891,7 @@
         <v>10</v>
       </c>
       <c r="F67">
-        <v>723</v>
+        <v>513</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
@@ -4911,7 +4911,7 @@
         <v>10</v>
       </c>
       <c r="F68">
-        <v>483</v>
+        <v>409</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
@@ -4931,7 +4931,7 @@
         <v>10</v>
       </c>
       <c r="F69">
-        <v>790</v>
+        <v>569</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
@@ -4951,7 +4951,7 @@
         <v>10</v>
       </c>
       <c r="F70">
-        <v>441</v>
+        <v>382</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
@@ -4971,7 +4971,7 @@
         <v>10</v>
       </c>
       <c r="F71">
-        <v>360</v>
+        <v>281</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
@@ -4991,7 +4991,7 @@
         <v>10</v>
       </c>
       <c r="F72">
-        <v>415</v>
+        <v>356</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
@@ -5011,7 +5011,7 @@
         <v>10</v>
       </c>
       <c r="F73">
-        <v>478</v>
+        <v>914</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
@@ -5031,7 +5031,7 @@
         <v>10</v>
       </c>
       <c r="F74">
-        <v>653</v>
+        <v>566</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
@@ -5051,7 +5051,7 @@
         <v>10</v>
       </c>
       <c r="F75">
-        <v>404</v>
+        <v>966</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
@@ -5071,7 +5071,7 @@
         <v>10</v>
       </c>
       <c r="F76">
-        <v>495</v>
+        <v>887</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
@@ -5091,7 +5091,7 @@
         <v>10</v>
       </c>
       <c r="F77">
-        <v>302</v>
+        <v>552</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
@@ -5111,7 +5111,7 @@
         <v>10</v>
       </c>
       <c r="F78">
-        <v>269</v>
+        <v>625</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
@@ -5131,7 +5131,7 @@
         <v>10</v>
       </c>
       <c r="F79">
-        <v>300</v>
+        <v>899</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
@@ -5151,7 +5151,7 @@
         <v>10</v>
       </c>
       <c r="F80">
-        <v>719</v>
+        <v>585</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
@@ -5171,7 +5171,7 @@
         <v>10</v>
       </c>
       <c r="F81">
-        <v>457</v>
+        <v>565</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
@@ -5191,7 +5191,7 @@
         <v>10</v>
       </c>
       <c r="F82">
-        <v>479</v>
+        <v>914</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
@@ -5211,7 +5211,7 @@
         <v>10</v>
       </c>
       <c r="F83">
-        <v>837</v>
+        <v>709</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
@@ -5231,7 +5231,7 @@
         <v>10</v>
       </c>
       <c r="F84">
-        <v>661</v>
+        <v>382</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
@@ -5251,7 +5251,7 @@
         <v>10</v>
       </c>
       <c r="F85">
-        <v>908</v>
+        <v>574</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
@@ -5271,7 +5271,7 @@
         <v>10</v>
       </c>
       <c r="F86">
-        <v>346</v>
+        <v>922</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
@@ -5291,7 +5291,7 @@
         <v>10</v>
       </c>
       <c r="F87">
-        <v>703</v>
+        <v>769</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
@@ -5311,7 +5311,7 @@
         <v>10</v>
       </c>
       <c r="F88">
-        <v>990</v>
+        <v>504</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
@@ -5331,7 +5331,7 @@
         <v>10</v>
       </c>
       <c r="F89">
-        <v>338</v>
+        <v>554</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
@@ -5351,7 +5351,7 @@
         <v>10</v>
       </c>
       <c r="F90">
-        <v>778</v>
+        <v>910</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
@@ -5371,7 +5371,7 @@
         <v>10</v>
       </c>
       <c r="F91">
-        <v>255</v>
+        <v>293</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
@@ -5391,7 +5391,7 @@
         <v>10</v>
       </c>
       <c r="F92">
-        <v>266</v>
+        <v>785</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
@@ -5411,7 +5411,7 @@
         <v>10</v>
       </c>
       <c r="F93">
-        <v>411</v>
+        <v>747</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
@@ -5431,7 +5431,7 @@
         <v>10</v>
       </c>
       <c r="F94">
-        <v>911</v>
+        <v>471</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
@@ -5451,7 +5451,7 @@
         <v>10</v>
       </c>
       <c r="F95">
-        <v>445</v>
+        <v>885</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
@@ -5471,7 +5471,7 @@
         <v>10</v>
       </c>
       <c r="F96">
-        <v>220</v>
+        <v>946</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
@@ -5491,7 +5491,7 @@
         <v>10</v>
       </c>
       <c r="F97">
-        <v>655</v>
+        <v>616</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
@@ -5511,7 +5511,7 @@
         <v>10</v>
       </c>
       <c r="F98">
-        <v>279</v>
+        <v>514</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
@@ -5531,7 +5531,7 @@
         <v>10</v>
       </c>
       <c r="F99">
-        <v>536</v>
+        <v>950</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
@@ -5551,7 +5551,7 @@
         <v>10</v>
       </c>
       <c r="F100">
-        <v>558</v>
+        <v>904</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
@@ -5571,7 +5571,7 @@
         <v>10</v>
       </c>
       <c r="F101">
-        <v>507</v>
+        <v>434</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
@@ -5591,7 +5591,7 @@
         <v>10</v>
       </c>
       <c r="F102">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
@@ -5611,7 +5611,7 @@
         <v>10</v>
       </c>
       <c r="F103">
-        <v>684</v>
+        <v>390</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
@@ -5631,7 +5631,7 @@
         <v>10</v>
       </c>
       <c r="F104">
-        <v>342</v>
+        <v>798</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
@@ -5651,7 +5651,7 @@
         <v>10</v>
       </c>
       <c r="F105">
-        <v>968</v>
+        <v>834</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
@@ -5671,7 +5671,7 @@
         <v>10</v>
       </c>
       <c r="F106">
-        <v>901</v>
+        <v>880</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
@@ -5691,7 +5691,7 @@
         <v>10</v>
       </c>
       <c r="F107">
-        <v>311</v>
+        <v>430</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
@@ -5711,7 +5711,7 @@
         <v>10</v>
       </c>
       <c r="F108">
-        <v>838</v>
+        <v>767</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
@@ -5731,7 +5731,7 @@
         <v>10</v>
       </c>
       <c r="F109">
-        <v>687</v>
+        <v>711</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
@@ -5751,7 +5751,7 @@
         <v>10</v>
       </c>
       <c r="F110">
-        <v>672</v>
+        <v>642</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
@@ -5771,7 +5771,7 @@
         <v>10</v>
       </c>
       <c r="F111">
-        <v>785</v>
+        <v>947</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
@@ -5791,7 +5791,7 @@
         <v>10</v>
       </c>
       <c r="F112">
-        <v>414</v>
+        <v>232</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
@@ -5811,7 +5811,7 @@
         <v>10</v>
       </c>
       <c r="F113">
-        <v>459</v>
+        <v>359</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
@@ -5831,7 +5831,7 @@
         <v>10</v>
       </c>
       <c r="F114">
-        <v>947</v>
+        <v>351</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
@@ -5851,7 +5851,7 @@
         <v>10</v>
       </c>
       <c r="F115">
-        <v>523</v>
+        <v>833</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
@@ -5871,7 +5871,7 @@
         <v>10</v>
       </c>
       <c r="F116">
-        <v>899</v>
+        <v>916</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
@@ -5891,7 +5891,7 @@
         <v>10</v>
       </c>
       <c r="F117">
-        <v>221</v>
+        <v>877</v>
       </c>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
@@ -5911,7 +5911,7 @@
         <v>10</v>
       </c>
       <c r="F118">
-        <v>744</v>
+        <v>260</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
@@ -5931,7 +5931,7 @@
         <v>10</v>
       </c>
       <c r="F119">
-        <v>408</v>
+        <v>381</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
@@ -5951,7 +5951,7 @@
         <v>10</v>
       </c>
       <c r="F120">
-        <v>520</v>
+        <v>945</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
@@ -5971,7 +5971,7 @@
         <v>10</v>
       </c>
       <c r="F121">
-        <v>265</v>
+        <v>917</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
@@ -5991,7 +5991,7 @@
         <v>10</v>
       </c>
       <c r="F122">
-        <v>253</v>
+        <v>719</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
@@ -6011,7 +6011,7 @@
         <v>10</v>
       </c>
       <c r="F123">
-        <v>867</v>
+        <v>939</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
@@ -6031,7 +6031,7 @@
         <v>10</v>
       </c>
       <c r="F124">
-        <v>281</v>
+        <v>983</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
@@ -6051,7 +6051,7 @@
         <v>10</v>
       </c>
       <c r="F125">
-        <v>776</v>
+        <v>612</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
@@ -6071,7 +6071,7 @@
         <v>10</v>
       </c>
       <c r="F126">
-        <v>786</v>
+        <v>551</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
@@ -6091,7 +6091,7 @@
         <v>10</v>
       </c>
       <c r="F127">
-        <v>566</v>
+        <v>806</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
@@ -6111,7 +6111,7 @@
         <v>10</v>
       </c>
       <c r="F128">
-        <v>444</v>
+        <v>312</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
@@ -6131,7 +6131,7 @@
         <v>10</v>
       </c>
       <c r="F129">
-        <v>448</v>
+        <v>435</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
@@ -6151,7 +6151,7 @@
         <v>10</v>
       </c>
       <c r="F130">
-        <v>685</v>
+        <v>526</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
@@ -6171,7 +6171,7 @@
         <v>10</v>
       </c>
       <c r="F131">
-        <v>747</v>
+        <v>338</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
@@ -6191,7 +6191,7 @@
         <v>10</v>
       </c>
       <c r="F132">
-        <v>613</v>
+        <v>508</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.25">
@@ -6211,7 +6211,7 @@
         <v>10</v>
       </c>
       <c r="F133">
-        <v>493</v>
+        <v>613</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.25">
@@ -6231,7 +6231,7 @@
         <v>10</v>
       </c>
       <c r="F134">
-        <v>337</v>
+        <v>874</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.25">
@@ -6251,7 +6251,7 @@
         <v>10</v>
       </c>
       <c r="F135">
-        <v>754</v>
+        <v>784</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.25">
@@ -6271,7 +6271,7 @@
         <v>10</v>
       </c>
       <c r="F136">
-        <v>778</v>
+        <v>894</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.25">
@@ -6291,7 +6291,7 @@
         <v>10</v>
       </c>
       <c r="F137">
-        <v>689</v>
+        <v>521</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.25">
@@ -6311,7 +6311,7 @@
         <v>10</v>
       </c>
       <c r="F138">
-        <v>870</v>
+        <v>622</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.25">
@@ -6331,7 +6331,7 @@
         <v>10</v>
       </c>
       <c r="F139">
-        <v>643</v>
+        <v>722</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.25">
@@ -6351,7 +6351,7 @@
         <v>10</v>
       </c>
       <c r="F140">
-        <v>943</v>
+        <v>743</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.25">
@@ -6371,7 +6371,7 @@
         <v>10</v>
       </c>
       <c r="F141">
-        <v>854</v>
+        <v>497</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.25">
@@ -6391,7 +6391,7 @@
         <v>10</v>
       </c>
       <c r="F142">
-        <v>989</v>
+        <v>999</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.25">
@@ -6411,7 +6411,7 @@
         <v>10</v>
       </c>
       <c r="F143">
-        <v>643</v>
+        <v>553</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.25">
@@ -6431,7 +6431,7 @@
         <v>10</v>
       </c>
       <c r="F144">
-        <v>786</v>
+        <v>536</v>
       </c>
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.25">
@@ -6451,7 +6451,7 @@
         <v>10</v>
       </c>
       <c r="F145">
-        <v>556</v>
+        <v>570</v>
       </c>
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.25">
@@ -6471,7 +6471,7 @@
         <v>10</v>
       </c>
       <c r="F146">
-        <v>796</v>
+        <v>771</v>
       </c>
     </row>
     <row r="147" spans="1:6" x14ac:dyDescent="0.25">
@@ -6491,7 +6491,7 @@
         <v>10</v>
       </c>
       <c r="F147">
-        <v>790</v>
+        <v>681</v>
       </c>
     </row>
     <row r="148" spans="1:6" x14ac:dyDescent="0.25">
@@ -6511,7 +6511,7 @@
         <v>10</v>
       </c>
       <c r="F148">
-        <v>987</v>
+        <v>427</v>
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.25">
@@ -6531,7 +6531,7 @@
         <v>10</v>
       </c>
       <c r="F149">
-        <v>724</v>
+        <v>520</v>
       </c>
     </row>
     <row r="150" spans="1:6" x14ac:dyDescent="0.25">
@@ -6551,7 +6551,7 @@
         <v>10</v>
       </c>
       <c r="F150">
-        <v>380</v>
+        <v>362</v>
       </c>
     </row>
     <row r="151" spans="1:6" x14ac:dyDescent="0.25">
@@ -6571,7 +6571,7 @@
         <v>10</v>
       </c>
       <c r="F151">
-        <v>244</v>
+        <v>202</v>
       </c>
     </row>
     <row r="152" spans="1:6" x14ac:dyDescent="0.25">
@@ -6591,7 +6591,7 @@
         <v>10</v>
       </c>
       <c r="F152">
-        <v>714</v>
+        <v>431</v>
       </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.25">
@@ -6611,7 +6611,7 @@
         <v>10</v>
       </c>
       <c r="F153">
-        <v>298</v>
+        <v>849</v>
       </c>
     </row>
     <row r="154" spans="1:6" x14ac:dyDescent="0.25">
@@ -6631,7 +6631,7 @@
         <v>10</v>
       </c>
       <c r="F154">
-        <v>278</v>
+        <v>673</v>
       </c>
     </row>
     <row r="155" spans="1:6" x14ac:dyDescent="0.25">
@@ -6651,7 +6651,7 @@
         <v>10</v>
       </c>
       <c r="F155">
-        <v>838</v>
+        <v>982</v>
       </c>
     </row>
     <row r="156" spans="1:6" x14ac:dyDescent="0.25">
@@ -6671,7 +6671,7 @@
         <v>10</v>
       </c>
       <c r="F156">
-        <v>577</v>
+        <v>683</v>
       </c>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.25">
@@ -6691,7 +6691,7 @@
         <v>10</v>
       </c>
       <c r="F157">
-        <v>632</v>
+        <v>670</v>
       </c>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.25">
@@ -6711,7 +6711,7 @@
         <v>10</v>
       </c>
       <c r="F158">
-        <v>444</v>
+        <v>278</v>
       </c>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.25">
@@ -6731,7 +6731,7 @@
         <v>10</v>
       </c>
       <c r="F159">
-        <v>668</v>
+        <v>599</v>
       </c>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.25">
@@ -6751,7 +6751,7 @@
         <v>10</v>
       </c>
       <c r="F160">
-        <v>457</v>
+        <v>405</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.25">
@@ -6771,7 +6771,7 @@
         <v>10</v>
       </c>
       <c r="F161">
-        <v>467</v>
+        <v>259</v>
       </c>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.25">
@@ -6791,7 +6791,7 @@
         <v>10</v>
       </c>
       <c r="F162">
-        <v>214</v>
+        <v>303</v>
       </c>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.25">
@@ -6811,7 +6811,7 @@
         <v>10</v>
       </c>
       <c r="F163">
-        <v>881</v>
+        <v>671</v>
       </c>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.25">
@@ -6831,7 +6831,7 @@
         <v>10</v>
       </c>
       <c r="F164">
-        <v>992</v>
+        <v>827</v>
       </c>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.25">
@@ -6851,7 +6851,7 @@
         <v>10</v>
       </c>
       <c r="F165">
-        <v>829</v>
+        <v>258</v>
       </c>
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.25">
@@ -6871,7 +6871,7 @@
         <v>10</v>
       </c>
       <c r="F166">
-        <v>222</v>
+        <v>231</v>
       </c>
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.25">
@@ -6891,7 +6891,7 @@
         <v>10</v>
       </c>
       <c r="F167">
-        <v>583</v>
+        <v>494</v>
       </c>
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.25">
@@ -6911,7 +6911,7 @@
         <v>10</v>
       </c>
       <c r="F168">
-        <v>900</v>
+        <v>807</v>
       </c>
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.25">
@@ -6931,7 +6931,7 @@
         <v>10</v>
       </c>
       <c r="F169">
-        <v>727</v>
+        <v>482</v>
       </c>
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.25">
@@ -6951,7 +6951,7 @@
         <v>10</v>
       </c>
       <c r="F170">
-        <v>686</v>
+        <v>356</v>
       </c>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.25">
@@ -6971,7 +6971,7 @@
         <v>10</v>
       </c>
       <c r="F171">
-        <v>237</v>
+        <v>443</v>
       </c>
     </row>
     <row r="172" spans="1:6" x14ac:dyDescent="0.25">
@@ -6991,7 +6991,7 @@
         <v>10</v>
       </c>
       <c r="F172">
-        <v>867</v>
+        <v>294</v>
       </c>
     </row>
     <row r="173" spans="1:6" x14ac:dyDescent="0.25">
@@ -7011,7 +7011,7 @@
         <v>10</v>
       </c>
       <c r="F173">
-        <v>397</v>
+        <v>723</v>
       </c>
     </row>
     <row r="174" spans="1:6" x14ac:dyDescent="0.25">
@@ -7031,7 +7031,7 @@
         <v>10</v>
       </c>
       <c r="F174">
-        <v>868</v>
+        <v>620</v>
       </c>
     </row>
     <row r="175" spans="1:6" x14ac:dyDescent="0.25">
@@ -7051,7 +7051,7 @@
         <v>10</v>
       </c>
       <c r="F175">
-        <v>336</v>
+        <v>567</v>
       </c>
     </row>
     <row r="176" spans="1:6" x14ac:dyDescent="0.25">
@@ -7071,7 +7071,7 @@
         <v>10</v>
       </c>
       <c r="F176">
-        <v>572</v>
+        <v>616</v>
       </c>
     </row>
     <row r="177" spans="1:6" x14ac:dyDescent="0.25">
@@ -7091,7 +7091,7 @@
         <v>10</v>
       </c>
       <c r="F177">
-        <v>398</v>
+        <v>377</v>
       </c>
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.25">
@@ -7111,7 +7111,7 @@
         <v>10</v>
       </c>
       <c r="F178">
-        <v>394</v>
+        <v>870</v>
       </c>
     </row>
     <row r="179" spans="1:6" x14ac:dyDescent="0.25">
@@ -7131,7 +7131,7 @@
         <v>10</v>
       </c>
       <c r="F179">
-        <v>832</v>
+        <v>463</v>
       </c>
     </row>
     <row r="180" spans="1:6" x14ac:dyDescent="0.25">
@@ -7151,7 +7151,7 @@
         <v>10</v>
       </c>
       <c r="F180">
-        <v>397</v>
+        <v>522</v>
       </c>
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.25">
@@ -7171,7 +7171,7 @@
         <v>10</v>
       </c>
       <c r="F181">
-        <v>494</v>
+        <v>365</v>
       </c>
     </row>
     <row r="182" spans="1:6" x14ac:dyDescent="0.25">
@@ -7191,7 +7191,7 @@
         <v>10</v>
       </c>
       <c r="F182">
-        <v>457</v>
+        <v>211</v>
       </c>
     </row>
     <row r="183" spans="1:6" x14ac:dyDescent="0.25">
@@ -7211,7 +7211,7 @@
         <v>10</v>
       </c>
       <c r="F183">
-        <v>596</v>
+        <v>685</v>
       </c>
     </row>
     <row r="184" spans="1:6" x14ac:dyDescent="0.25">
@@ -7231,7 +7231,7 @@
         <v>10</v>
       </c>
       <c r="F184">
-        <v>613</v>
+        <v>253</v>
       </c>
     </row>
     <row r="185" spans="1:6" x14ac:dyDescent="0.25">
@@ -7251,7 +7251,7 @@
         <v>10</v>
       </c>
       <c r="F185">
-        <v>294</v>
+        <v>674</v>
       </c>
     </row>
     <row r="186" spans="1:6" x14ac:dyDescent="0.25">
@@ -7271,7 +7271,7 @@
         <v>10</v>
       </c>
       <c r="F186">
-        <v>527</v>
+        <v>258</v>
       </c>
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.25">
@@ -7291,7 +7291,7 @@
         <v>10</v>
       </c>
       <c r="F187">
-        <v>659</v>
+        <v>402</v>
       </c>
     </row>
     <row r="188" spans="1:6" x14ac:dyDescent="0.25">
@@ -7311,7 +7311,7 @@
         <v>10</v>
       </c>
       <c r="F188">
-        <v>962</v>
+        <v>784</v>
       </c>
     </row>
     <row r="189" spans="1:6" x14ac:dyDescent="0.25">
@@ -7331,7 +7331,7 @@
         <v>10</v>
       </c>
       <c r="F189">
-        <v>499</v>
+        <v>205</v>
       </c>
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.25">
@@ -7351,7 +7351,7 @@
         <v>10</v>
       </c>
       <c r="F190">
-        <v>255</v>
+        <v>771</v>
       </c>
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.25">
@@ -7371,7 +7371,7 @@
         <v>10</v>
       </c>
       <c r="F191">
-        <v>384</v>
+        <v>415</v>
       </c>
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.25">
@@ -7391,7 +7391,7 @@
         <v>10</v>
       </c>
       <c r="F192">
-        <v>431</v>
+        <v>406</v>
       </c>
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.25">
@@ -7411,7 +7411,7 @@
         <v>10</v>
       </c>
       <c r="F193">
-        <v>887</v>
+        <v>483</v>
       </c>
     </row>
     <row r="194" spans="1:6" x14ac:dyDescent="0.25">
@@ -7431,7 +7431,7 @@
         <v>10</v>
       </c>
       <c r="F194">
-        <v>858</v>
+        <v>399</v>
       </c>
     </row>
     <row r="195" spans="1:6" x14ac:dyDescent="0.25">
@@ -7451,7 +7451,7 @@
         <v>10</v>
       </c>
       <c r="F195">
-        <v>452</v>
+        <v>936</v>
       </c>
     </row>
     <row r="196" spans="1:6" x14ac:dyDescent="0.25">
@@ -7471,7 +7471,7 @@
         <v>10</v>
       </c>
       <c r="F196">
-        <v>886</v>
+        <v>978</v>
       </c>
     </row>
     <row r="197" spans="1:6" x14ac:dyDescent="0.25">
@@ -7491,7 +7491,7 @@
         <v>10</v>
       </c>
       <c r="F197">
-        <v>958</v>
+        <v>920</v>
       </c>
     </row>
     <row r="198" spans="1:6" x14ac:dyDescent="0.25">
@@ -7511,7 +7511,7 @@
         <v>10</v>
       </c>
       <c r="F198">
-        <v>360</v>
+        <v>431</v>
       </c>
     </row>
     <row r="199" spans="1:6" x14ac:dyDescent="0.25">
@@ -7531,7 +7531,7 @@
         <v>10</v>
       </c>
       <c r="F199">
-        <v>449</v>
+        <v>957</v>
       </c>
     </row>
     <row r="200" spans="1:6" x14ac:dyDescent="0.25">
@@ -7551,7 +7551,7 @@
         <v>10</v>
       </c>
       <c r="F200">
-        <v>832</v>
+        <v>248</v>
       </c>
     </row>
     <row r="201" spans="1:6" x14ac:dyDescent="0.25">
@@ -7571,7 +7571,7 @@
         <v>10</v>
       </c>
       <c r="F201">
-        <v>939</v>
+        <v>559</v>
       </c>
     </row>
     <row r="202" spans="1:6" x14ac:dyDescent="0.25">
@@ -7591,7 +7591,7 @@
         <v>10</v>
       </c>
       <c r="F202">
-        <v>310</v>
+        <v>587</v>
       </c>
     </row>
     <row r="203" spans="1:6" x14ac:dyDescent="0.25">
@@ -7611,7 +7611,7 @@
         <v>10</v>
       </c>
       <c r="F203">
-        <v>285</v>
+        <v>444</v>
       </c>
     </row>
     <row r="204" spans="1:6" x14ac:dyDescent="0.25">
@@ -7631,7 +7631,7 @@
         <v>10</v>
       </c>
       <c r="F204">
-        <v>637</v>
+        <v>261</v>
       </c>
     </row>
     <row r="205" spans="1:6" x14ac:dyDescent="0.25">
@@ -7651,7 +7651,7 @@
         <v>10</v>
       </c>
       <c r="F205">
-        <v>687</v>
+        <v>292</v>
       </c>
     </row>
     <row r="206" spans="1:6" x14ac:dyDescent="0.25">
@@ -7671,7 +7671,7 @@
         <v>10</v>
       </c>
       <c r="F206">
-        <v>382</v>
+        <v>837</v>
       </c>
     </row>
     <row r="207" spans="1:6" x14ac:dyDescent="0.25">
@@ -7691,7 +7691,7 @@
         <v>10</v>
       </c>
       <c r="F207">
-        <v>961</v>
+        <v>530</v>
       </c>
     </row>
     <row r="208" spans="1:6" x14ac:dyDescent="0.25">
@@ -7711,7 +7711,7 @@
         <v>10</v>
       </c>
       <c r="F208">
-        <v>279</v>
+        <v>803</v>
       </c>
     </row>
     <row r="209" spans="1:6" x14ac:dyDescent="0.25">
@@ -7731,7 +7731,7 @@
         <v>10</v>
       </c>
       <c r="F209">
-        <v>276</v>
+        <v>922</v>
       </c>
     </row>
     <row r="210" spans="1:6" x14ac:dyDescent="0.25">
@@ -7751,7 +7751,7 @@
         <v>10</v>
       </c>
       <c r="F210">
-        <v>801</v>
+        <v>511</v>
       </c>
     </row>
     <row r="211" spans="1:6" x14ac:dyDescent="0.25">
@@ -7771,7 +7771,7 @@
         <v>10</v>
       </c>
       <c r="F211">
-        <v>534</v>
+        <v>442</v>
       </c>
     </row>
     <row r="212" spans="1:6" x14ac:dyDescent="0.25">
@@ -7791,7 +7791,7 @@
         <v>10</v>
       </c>
       <c r="F212">
-        <v>857</v>
+        <v>231</v>
       </c>
     </row>
     <row r="213" spans="1:6" x14ac:dyDescent="0.25">
@@ -7811,7 +7811,7 @@
         <v>10</v>
       </c>
       <c r="F213">
-        <v>820</v>
+        <v>616</v>
       </c>
     </row>
     <row r="214" spans="1:6" x14ac:dyDescent="0.25">
@@ -7831,7 +7831,7 @@
         <v>10</v>
       </c>
       <c r="F214">
-        <v>799</v>
+        <v>660</v>
       </c>
     </row>
     <row r="215" spans="1:6" x14ac:dyDescent="0.25">
@@ -7851,7 +7851,7 @@
         <v>10</v>
       </c>
       <c r="F215">
-        <v>573</v>
+        <v>553</v>
       </c>
     </row>
     <row r="216" spans="1:6" x14ac:dyDescent="0.25">
@@ -7871,7 +7871,7 @@
         <v>10</v>
       </c>
       <c r="F216">
-        <v>599</v>
+        <v>230</v>
       </c>
     </row>
     <row r="217" spans="1:6" x14ac:dyDescent="0.25">
@@ -7891,7 +7891,7 @@
         <v>10</v>
       </c>
       <c r="F217">
-        <v>435</v>
+        <v>413</v>
       </c>
     </row>
     <row r="218" spans="1:6" x14ac:dyDescent="0.25">
@@ -7911,7 +7911,7 @@
         <v>10</v>
       </c>
       <c r="F218">
-        <v>596</v>
+        <v>620</v>
       </c>
     </row>
     <row r="219" spans="1:6" x14ac:dyDescent="0.25">
@@ -7931,7 +7931,7 @@
         <v>10</v>
       </c>
       <c r="F219">
-        <v>215</v>
+        <v>208</v>
       </c>
     </row>
     <row r="220" spans="1:6" x14ac:dyDescent="0.25">
@@ -7951,7 +7951,7 @@
         <v>10</v>
       </c>
       <c r="F220">
-        <v>612</v>
+        <v>332</v>
       </c>
     </row>
     <row r="221" spans="1:6" x14ac:dyDescent="0.25">
@@ -7971,7 +7971,7 @@
         <v>10</v>
       </c>
       <c r="F221">
-        <v>763</v>
+        <v>342</v>
       </c>
     </row>
     <row r="222" spans="1:6" x14ac:dyDescent="0.25">
@@ -7991,7 +7991,7 @@
         <v>10</v>
       </c>
       <c r="F222">
-        <v>517</v>
+        <v>479</v>
       </c>
     </row>
     <row r="223" spans="1:6" x14ac:dyDescent="0.25">
@@ -8011,7 +8011,7 @@
         <v>10</v>
       </c>
       <c r="F223">
-        <v>782</v>
+        <v>207</v>
       </c>
     </row>
     <row r="224" spans="1:6" x14ac:dyDescent="0.25">
@@ -8031,7 +8031,7 @@
         <v>10</v>
       </c>
       <c r="F224">
-        <v>777</v>
+        <v>788</v>
       </c>
     </row>
     <row r="225" spans="1:6" x14ac:dyDescent="0.25">
@@ -8051,7 +8051,7 @@
         <v>10</v>
       </c>
       <c r="F225">
-        <v>399</v>
+        <v>425</v>
       </c>
     </row>
     <row r="226" spans="1:6" x14ac:dyDescent="0.25">
@@ -8071,7 +8071,7 @@
         <v>10</v>
       </c>
       <c r="F226">
-        <v>964</v>
+        <v>776</v>
       </c>
     </row>
     <row r="227" spans="1:6" x14ac:dyDescent="0.25">
@@ -8091,7 +8091,7 @@
         <v>10</v>
       </c>
       <c r="F227">
-        <v>398</v>
+        <v>959</v>
       </c>
     </row>
     <row r="228" spans="1:6" x14ac:dyDescent="0.25">
@@ -8111,7 +8111,7 @@
         <v>10</v>
       </c>
       <c r="F228">
-        <v>750</v>
+        <v>831</v>
       </c>
     </row>
     <row r="229" spans="1:6" x14ac:dyDescent="0.25">
@@ -8131,7 +8131,7 @@
         <v>10</v>
       </c>
       <c r="F229">
-        <v>911</v>
+        <v>868</v>
       </c>
     </row>
     <row r="230" spans="1:6" x14ac:dyDescent="0.25">
@@ -8151,7 +8151,7 @@
         <v>10</v>
       </c>
       <c r="F230">
-        <v>392</v>
+        <v>571</v>
       </c>
     </row>
     <row r="231" spans="1:6" x14ac:dyDescent="0.25">
@@ -8171,7 +8171,7 @@
         <v>10</v>
       </c>
       <c r="F231">
-        <v>308</v>
+        <v>467</v>
       </c>
     </row>
     <row r="232" spans="1:6" x14ac:dyDescent="0.25">
@@ -8191,7 +8191,7 @@
         <v>10</v>
       </c>
       <c r="F232">
-        <v>534</v>
+        <v>750</v>
       </c>
     </row>
     <row r="233" spans="1:6" x14ac:dyDescent="0.25">
@@ -8211,7 +8211,7 @@
         <v>10</v>
       </c>
       <c r="F233">
-        <v>451</v>
+        <v>297</v>
       </c>
     </row>
     <row r="234" spans="1:6" x14ac:dyDescent="0.25">
@@ -8231,7 +8231,7 @@
         <v>10</v>
       </c>
       <c r="F234">
-        <v>665</v>
+        <v>328</v>
       </c>
     </row>
     <row r="235" spans="1:6" x14ac:dyDescent="0.25">
@@ -8251,7 +8251,7 @@
         <v>10</v>
       </c>
       <c r="F235">
-        <v>391</v>
+        <v>829</v>
       </c>
     </row>
     <row r="236" spans="1:6" x14ac:dyDescent="0.25">
@@ -8271,7 +8271,7 @@
         <v>10</v>
       </c>
       <c r="F236">
-        <v>666</v>
+        <v>950</v>
       </c>
     </row>
     <row r="237" spans="1:6" x14ac:dyDescent="0.25">
@@ -8291,7 +8291,7 @@
         <v>10</v>
       </c>
       <c r="F237">
-        <v>770</v>
+        <v>847</v>
       </c>
     </row>
     <row r="238" spans="1:6" x14ac:dyDescent="0.25">
@@ -8311,7 +8311,7 @@
         <v>10</v>
       </c>
       <c r="F238">
-        <v>718</v>
+        <v>967</v>
       </c>
     </row>
     <row r="239" spans="1:6" x14ac:dyDescent="0.25">
@@ -8331,7 +8331,7 @@
         <v>10</v>
       </c>
       <c r="F239">
-        <v>613</v>
+        <v>968</v>
       </c>
     </row>
     <row r="240" spans="1:6" x14ac:dyDescent="0.25">
@@ -8351,7 +8351,7 @@
         <v>10</v>
       </c>
       <c r="F240">
-        <v>767</v>
+        <v>759</v>
       </c>
     </row>
     <row r="241" spans="1:6" x14ac:dyDescent="0.25">
@@ -8371,7 +8371,7 @@
         <v>10</v>
       </c>
       <c r="F241">
-        <v>493</v>
+        <v>889</v>
       </c>
     </row>
     <row r="242" spans="1:6" x14ac:dyDescent="0.25">
@@ -8391,7 +8391,7 @@
         <v>10</v>
       </c>
       <c r="F242">
-        <v>518</v>
+        <v>281</v>
       </c>
     </row>
     <row r="243" spans="1:6" x14ac:dyDescent="0.25">
@@ -8411,7 +8411,7 @@
         <v>10</v>
       </c>
       <c r="F243">
-        <v>822</v>
+        <v>689</v>
       </c>
     </row>
     <row r="244" spans="1:6" x14ac:dyDescent="0.25">
@@ -8431,7 +8431,7 @@
         <v>10</v>
       </c>
       <c r="F244">
-        <v>630</v>
+        <v>857</v>
       </c>
     </row>
     <row r="245" spans="1:6" x14ac:dyDescent="0.25">
@@ -8451,7 +8451,7 @@
         <v>10</v>
       </c>
       <c r="F245">
-        <v>862</v>
+        <v>293</v>
       </c>
     </row>
     <row r="246" spans="1:6" x14ac:dyDescent="0.25">
@@ -8471,7 +8471,7 @@
         <v>10</v>
       </c>
       <c r="F246">
-        <v>296</v>
+        <v>558</v>
       </c>
     </row>
     <row r="247" spans="1:6" x14ac:dyDescent="0.25">
@@ -8491,7 +8491,7 @@
         <v>10</v>
       </c>
       <c r="F247">
-        <v>806</v>
+        <v>903</v>
       </c>
     </row>
     <row r="248" spans="1:6" x14ac:dyDescent="0.25">
@@ -8511,7 +8511,7 @@
         <v>10</v>
       </c>
       <c r="F248">
-        <v>484</v>
+        <v>268</v>
       </c>
     </row>
     <row r="249" spans="1:6" x14ac:dyDescent="0.25">
@@ -8531,7 +8531,7 @@
         <v>10</v>
       </c>
       <c r="F249">
-        <v>720</v>
+        <v>528</v>
       </c>
     </row>
     <row r="250" spans="1:6" x14ac:dyDescent="0.25">
@@ -8551,7 +8551,7 @@
         <v>10</v>
       </c>
       <c r="F250">
-        <v>590</v>
+        <v>734</v>
       </c>
     </row>
     <row r="251" spans="1:6" x14ac:dyDescent="0.25">
@@ -8571,7 +8571,7 @@
         <v>10</v>
       </c>
       <c r="F251">
-        <v>468</v>
+        <v>229</v>
       </c>
     </row>
     <row r="252" spans="1:6" x14ac:dyDescent="0.25">
@@ -8591,7 +8591,7 @@
         <v>10</v>
       </c>
       <c r="F252">
-        <v>333</v>
+        <v>601</v>
       </c>
     </row>
     <row r="253" spans="1:6" x14ac:dyDescent="0.25">
@@ -8611,7 +8611,7 @@
         <v>10</v>
       </c>
       <c r="F253">
-        <v>327</v>
+        <v>683</v>
       </c>
     </row>
     <row r="254" spans="1:6" x14ac:dyDescent="0.25">
@@ -8631,7 +8631,7 @@
         <v>10</v>
       </c>
       <c r="F254">
-        <v>609</v>
+        <v>922</v>
       </c>
     </row>
     <row r="255" spans="1:6" x14ac:dyDescent="0.25">
@@ -8651,7 +8651,7 @@
         <v>10</v>
       </c>
       <c r="F255">
-        <v>638</v>
+        <v>946</v>
       </c>
     </row>
     <row r="256" spans="1:6" x14ac:dyDescent="0.25">
@@ -8671,7 +8671,7 @@
         <v>10</v>
       </c>
       <c r="F256">
-        <v>306</v>
+        <v>780</v>
       </c>
     </row>
     <row r="257" spans="1:6" x14ac:dyDescent="0.25">
@@ -8691,7 +8691,7 @@
         <v>10</v>
       </c>
       <c r="F257">
-        <v>657</v>
+        <v>514</v>
       </c>
     </row>
     <row r="258" spans="1:6" x14ac:dyDescent="0.25">
@@ -8711,7 +8711,7 @@
         <v>10</v>
       </c>
       <c r="F258">
-        <v>305</v>
+        <v>205</v>
       </c>
     </row>
     <row r="259" spans="1:6" x14ac:dyDescent="0.25">
@@ -8731,7 +8731,7 @@
         <v>10</v>
       </c>
       <c r="F259">
-        <v>594</v>
+        <v>682</v>
       </c>
     </row>
     <row r="260" spans="1:6" x14ac:dyDescent="0.25">
@@ -8751,7 +8751,7 @@
         <v>10</v>
       </c>
       <c r="F260">
-        <v>927</v>
+        <v>433</v>
       </c>
     </row>
     <row r="261" spans="1:6" x14ac:dyDescent="0.25">
@@ -8771,7 +8771,7 @@
         <v>10</v>
       </c>
       <c r="F261">
-        <v>746</v>
+        <v>691</v>
       </c>
     </row>
     <row r="262" spans="1:6" x14ac:dyDescent="0.25">
@@ -8791,7 +8791,7 @@
         <v>10</v>
       </c>
       <c r="F262">
-        <v>771</v>
+        <v>725</v>
       </c>
     </row>
     <row r="263" spans="1:6" x14ac:dyDescent="0.25">
@@ -8811,7 +8811,7 @@
         <v>10</v>
       </c>
       <c r="F263">
-        <v>307</v>
+        <v>303</v>
       </c>
     </row>
     <row r="264" spans="1:6" x14ac:dyDescent="0.25">
@@ -8831,7 +8831,7 @@
         <v>10</v>
       </c>
       <c r="F264">
-        <v>998</v>
+        <v>830</v>
       </c>
     </row>
     <row r="265" spans="1:6" x14ac:dyDescent="0.25">
@@ -8851,7 +8851,7 @@
         <v>10</v>
       </c>
       <c r="F265">
-        <v>723</v>
+        <v>987</v>
       </c>
     </row>
     <row r="266" spans="1:6" x14ac:dyDescent="0.25">
@@ -8871,7 +8871,7 @@
         <v>10</v>
       </c>
       <c r="F266">
-        <v>214</v>
+        <v>947</v>
       </c>
     </row>
     <row r="267" spans="1:6" x14ac:dyDescent="0.25">
@@ -8891,7 +8891,7 @@
         <v>10</v>
       </c>
       <c r="F267">
-        <v>579</v>
+        <v>970</v>
       </c>
     </row>
     <row r="268" spans="1:6" x14ac:dyDescent="0.25">
@@ -8911,7 +8911,7 @@
         <v>10</v>
       </c>
       <c r="F268">
-        <v>564</v>
+        <v>737</v>
       </c>
     </row>
     <row r="269" spans="1:6" x14ac:dyDescent="0.25">
@@ -8931,7 +8931,7 @@
         <v>10</v>
       </c>
       <c r="F269">
-        <v>636</v>
+        <v>394</v>
       </c>
     </row>
     <row r="270" spans="1:6" x14ac:dyDescent="0.25">
@@ -8951,7 +8951,7 @@
         <v>10</v>
       </c>
       <c r="F270">
-        <v>547</v>
+        <v>861</v>
       </c>
     </row>
     <row r="271" spans="1:6" x14ac:dyDescent="0.25">
@@ -8971,7 +8971,7 @@
         <v>10</v>
       </c>
       <c r="F271">
-        <v>933</v>
+        <v>468</v>
       </c>
     </row>
     <row r="272" spans="1:6" x14ac:dyDescent="0.25">
@@ -8991,7 +8991,7 @@
         <v>10</v>
       </c>
       <c r="F272">
-        <v>996</v>
+        <v>669</v>
       </c>
     </row>
     <row r="273" spans="1:6" x14ac:dyDescent="0.25">
@@ -9011,7 +9011,7 @@
         <v>10</v>
       </c>
       <c r="F273">
-        <v>749</v>
+        <v>396</v>
       </c>
     </row>
     <row r="274" spans="1:6" x14ac:dyDescent="0.25">
@@ -9031,7 +9031,7 @@
         <v>10</v>
       </c>
       <c r="F274">
-        <v>995</v>
+        <v>449</v>
       </c>
     </row>
     <row r="275" spans="1:6" x14ac:dyDescent="0.25">
@@ -9051,7 +9051,7 @@
         <v>10</v>
       </c>
       <c r="F275">
-        <v>747</v>
+        <v>478</v>
       </c>
     </row>
     <row r="276" spans="1:6" x14ac:dyDescent="0.25">
@@ -9071,7 +9071,7 @@
         <v>10</v>
       </c>
       <c r="F276">
-        <v>465</v>
+        <v>544</v>
       </c>
     </row>
     <row r="277" spans="1:6" x14ac:dyDescent="0.25">
@@ -9091,7 +9091,7 @@
         <v>10</v>
       </c>
       <c r="F277">
-        <v>892</v>
+        <v>222</v>
       </c>
     </row>
     <row r="278" spans="1:6" x14ac:dyDescent="0.25">
@@ -9111,7 +9111,7 @@
         <v>10</v>
       </c>
       <c r="F278">
-        <v>387</v>
+        <v>595</v>
       </c>
     </row>
     <row r="279" spans="1:6" x14ac:dyDescent="0.25">
@@ -9131,7 +9131,7 @@
         <v>10</v>
       </c>
       <c r="F279">
-        <v>543</v>
+        <v>983</v>
       </c>
     </row>
     <row r="280" spans="1:6" x14ac:dyDescent="0.25">
@@ -9151,7 +9151,7 @@
         <v>10</v>
       </c>
       <c r="F280">
-        <v>404</v>
+        <v>681</v>
       </c>
     </row>
     <row r="281" spans="1:6" x14ac:dyDescent="0.25">
@@ -9171,7 +9171,7 @@
         <v>10</v>
       </c>
       <c r="F281">
-        <v>651</v>
+        <v>268</v>
       </c>
     </row>
     <row r="282" spans="1:6" x14ac:dyDescent="0.25">
@@ -9191,7 +9191,7 @@
         <v>10</v>
       </c>
       <c r="F282">
-        <v>739</v>
+        <v>298</v>
       </c>
     </row>
     <row r="283" spans="1:6" x14ac:dyDescent="0.25">
@@ -9211,7 +9211,7 @@
         <v>10</v>
       </c>
       <c r="F283">
-        <v>825</v>
+        <v>770</v>
       </c>
     </row>
     <row r="284" spans="1:6" x14ac:dyDescent="0.25">
@@ -9231,7 +9231,7 @@
         <v>10</v>
       </c>
       <c r="F284">
-        <v>394</v>
+        <v>497</v>
       </c>
     </row>
     <row r="285" spans="1:6" x14ac:dyDescent="0.25">
@@ -9251,7 +9251,7 @@
         <v>10</v>
       </c>
       <c r="F285">
-        <v>656</v>
+        <v>862</v>
       </c>
     </row>
     <row r="286" spans="1:6" x14ac:dyDescent="0.25">
@@ -9271,7 +9271,7 @@
         <v>10</v>
       </c>
       <c r="F286">
-        <v>722</v>
+        <v>318</v>
       </c>
     </row>
     <row r="287" spans="1:6" x14ac:dyDescent="0.25">
@@ -9291,7 +9291,7 @@
         <v>10</v>
       </c>
       <c r="F287">
-        <v>712</v>
+        <v>732</v>
       </c>
     </row>
     <row r="288" spans="1:6" x14ac:dyDescent="0.25">
@@ -9311,7 +9311,7 @@
         <v>10</v>
       </c>
       <c r="F288">
-        <v>814</v>
+        <v>492</v>
       </c>
     </row>
     <row r="289" spans="1:6" x14ac:dyDescent="0.25">
@@ -9331,7 +9331,7 @@
         <v>10</v>
       </c>
       <c r="F289">
-        <v>602</v>
+        <v>367</v>
       </c>
     </row>
     <row r="290" spans="1:6" x14ac:dyDescent="0.25">
@@ -9351,7 +9351,7 @@
         <v>10</v>
       </c>
       <c r="F290">
-        <v>804</v>
+        <v>828</v>
       </c>
     </row>
     <row r="291" spans="1:6" x14ac:dyDescent="0.25">
@@ -9371,7 +9371,7 @@
         <v>10</v>
       </c>
       <c r="F291">
-        <v>967</v>
+        <v>344</v>
       </c>
     </row>
     <row r="292" spans="1:6" x14ac:dyDescent="0.25">
@@ -9391,7 +9391,7 @@
         <v>10</v>
       </c>
       <c r="F292">
-        <v>624</v>
+        <v>906</v>
       </c>
     </row>
     <row r="293" spans="1:6" x14ac:dyDescent="0.25">
@@ -9411,7 +9411,7 @@
         <v>10</v>
       </c>
       <c r="F293">
-        <v>358</v>
+        <v>384</v>
       </c>
     </row>
     <row r="294" spans="1:6" x14ac:dyDescent="0.25">
@@ -9431,7 +9431,7 @@
         <v>10</v>
       </c>
       <c r="F294">
-        <v>750</v>
+        <v>660</v>
       </c>
     </row>
     <row r="295" spans="1:6" x14ac:dyDescent="0.25">
@@ -9451,7 +9451,7 @@
         <v>10</v>
       </c>
       <c r="F295">
-        <v>622</v>
+        <v>755</v>
       </c>
     </row>
     <row r="296" spans="1:6" x14ac:dyDescent="0.25">
@@ -9471,7 +9471,7 @@
         <v>10</v>
       </c>
       <c r="F296">
-        <v>713</v>
+        <v>875</v>
       </c>
     </row>
     <row r="297" spans="1:6" x14ac:dyDescent="0.25">
@@ -9491,7 +9491,7 @@
         <v>10</v>
       </c>
       <c r="F297">
-        <v>815</v>
+        <v>252</v>
       </c>
     </row>
     <row r="298" spans="1:6" x14ac:dyDescent="0.25">
@@ -9511,7 +9511,7 @@
         <v>10</v>
       </c>
       <c r="F298">
-        <v>258</v>
+        <v>507</v>
       </c>
     </row>
     <row r="299" spans="1:6" x14ac:dyDescent="0.25">
@@ -9531,7 +9531,7 @@
         <v>10</v>
       </c>
       <c r="F299">
-        <v>417</v>
+        <v>591</v>
       </c>
     </row>
     <row r="300" spans="1:6" x14ac:dyDescent="0.25">
@@ -9551,7 +9551,7 @@
         <v>10</v>
       </c>
       <c r="F300">
-        <v>206</v>
+        <v>347</v>
       </c>
     </row>
     <row r="301" spans="1:6" x14ac:dyDescent="0.25">
@@ -9571,7 +9571,7 @@
         <v>10</v>
       </c>
       <c r="F301">
-        <v>201</v>
+        <v>584</v>
       </c>
     </row>
     <row r="302" spans="1:6" x14ac:dyDescent="0.25">
@@ -9591,7 +9591,7 @@
         <v>10</v>
       </c>
       <c r="F302">
-        <v>995</v>
+        <v>751</v>
       </c>
     </row>
     <row r="303" spans="1:6" x14ac:dyDescent="0.25">
@@ -9611,7 +9611,7 @@
         <v>10</v>
       </c>
       <c r="F303">
-        <v>292</v>
+        <v>822</v>
       </c>
     </row>
     <row r="304" spans="1:6" x14ac:dyDescent="0.25">
@@ -9631,7 +9631,7 @@
         <v>10</v>
       </c>
       <c r="F304">
-        <v>422</v>
+        <v>528</v>
       </c>
     </row>
     <row r="305" spans="1:6" x14ac:dyDescent="0.25">
@@ -9651,7 +9651,7 @@
         <v>10</v>
       </c>
       <c r="F305">
-        <v>714</v>
+        <v>773</v>
       </c>
     </row>
     <row r="306" spans="1:6" x14ac:dyDescent="0.25">
@@ -9671,7 +9671,7 @@
         <v>10</v>
       </c>
       <c r="F306">
-        <v>538</v>
+        <v>269</v>
       </c>
     </row>
     <row r="307" spans="1:6" x14ac:dyDescent="0.25">
@@ -9691,7 +9691,7 @@
         <v>10</v>
       </c>
       <c r="F307">
-        <v>313</v>
+        <v>304</v>
       </c>
     </row>
     <row r="308" spans="1:6" x14ac:dyDescent="0.25">
@@ -9711,7 +9711,7 @@
         <v>10</v>
       </c>
       <c r="F308">
-        <v>405</v>
+        <v>400</v>
       </c>
     </row>
     <row r="309" spans="1:6" x14ac:dyDescent="0.25">
@@ -9731,7 +9731,7 @@
         <v>10</v>
       </c>
       <c r="F309">
-        <v>839</v>
+        <v>345</v>
       </c>
     </row>
     <row r="310" spans="1:6" x14ac:dyDescent="0.25">
@@ -9751,7 +9751,7 @@
         <v>10</v>
       </c>
       <c r="F310">
-        <v>517</v>
+        <v>620</v>
       </c>
     </row>
     <row r="311" spans="1:6" x14ac:dyDescent="0.25">
@@ -9771,7 +9771,7 @@
         <v>10</v>
       </c>
       <c r="F311">
-        <v>904</v>
+        <v>719</v>
       </c>
     </row>
     <row r="312" spans="1:6" x14ac:dyDescent="0.25">
@@ -9791,7 +9791,7 @@
         <v>10</v>
       </c>
       <c r="F312">
-        <v>929</v>
+        <v>731</v>
       </c>
     </row>
     <row r="313" spans="1:6" x14ac:dyDescent="0.25">
@@ -9811,7 +9811,7 @@
         <v>10</v>
       </c>
       <c r="F313">
-        <v>997</v>
+        <v>257</v>
       </c>
     </row>
     <row r="314" spans="1:6" x14ac:dyDescent="0.25">
@@ -9831,7 +9831,7 @@
         <v>10</v>
       </c>
       <c r="F314">
-        <v>710</v>
+        <v>888</v>
       </c>
     </row>
     <row r="315" spans="1:6" x14ac:dyDescent="0.25">
@@ -9851,7 +9851,7 @@
         <v>10</v>
       </c>
       <c r="F315">
-        <v>583</v>
+        <v>767</v>
       </c>
     </row>
     <row r="316" spans="1:6" x14ac:dyDescent="0.25">
@@ -9871,7 +9871,7 @@
         <v>10</v>
       </c>
       <c r="F316">
-        <v>732</v>
+        <v>386</v>
       </c>
     </row>
     <row r="317" spans="1:6" x14ac:dyDescent="0.25">
@@ -9891,7 +9891,7 @@
         <v>10</v>
       </c>
       <c r="F317">
-        <v>340</v>
+        <v>253</v>
       </c>
     </row>
     <row r="318" spans="1:6" x14ac:dyDescent="0.25">
@@ -9911,7 +9911,7 @@
         <v>10</v>
       </c>
       <c r="F318">
-        <v>486</v>
+        <v>288</v>
       </c>
     </row>
     <row r="319" spans="1:6" x14ac:dyDescent="0.25">
@@ -9931,7 +9931,7 @@
         <v>10</v>
       </c>
       <c r="F319">
-        <v>601</v>
+        <v>946</v>
       </c>
     </row>
     <row r="320" spans="1:6" x14ac:dyDescent="0.25">
@@ -9951,7 +9951,7 @@
         <v>10</v>
       </c>
       <c r="F320">
-        <v>265</v>
+        <v>847</v>
       </c>
     </row>
     <row r="321" spans="1:6" x14ac:dyDescent="0.25">
@@ -9971,7 +9971,7 @@
         <v>10</v>
       </c>
       <c r="F321">
-        <v>864</v>
+        <v>390</v>
       </c>
     </row>
     <row r="322" spans="1:6" x14ac:dyDescent="0.25">
@@ -9991,7 +9991,7 @@
         <v>10</v>
       </c>
       <c r="F322">
-        <v>356</v>
+        <v>261</v>
       </c>
     </row>
     <row r="323" spans="1:6" x14ac:dyDescent="0.25">
@@ -10011,7 +10011,7 @@
         <v>10</v>
       </c>
       <c r="F323">
-        <v>307</v>
+        <v>371</v>
       </c>
     </row>
     <row r="324" spans="1:6" x14ac:dyDescent="0.25">
@@ -10031,7 +10031,7 @@
         <v>10</v>
       </c>
       <c r="F324">
-        <v>852</v>
+        <v>911</v>
       </c>
     </row>
     <row r="325" spans="1:6" x14ac:dyDescent="0.25">
@@ -10051,7 +10051,7 @@
         <v>10</v>
       </c>
       <c r="F325">
-        <v>207</v>
+        <v>950</v>
       </c>
     </row>
     <row r="326" spans="1:6" x14ac:dyDescent="0.25">
@@ -10071,7 +10071,7 @@
         <v>10</v>
       </c>
       <c r="F326">
-        <v>257</v>
+        <v>717</v>
       </c>
     </row>
     <row r="327" spans="1:6" x14ac:dyDescent="0.25">
@@ -10091,7 +10091,7 @@
         <v>10</v>
       </c>
       <c r="F327">
-        <v>205</v>
+        <v>228</v>
       </c>
     </row>
     <row r="328" spans="1:6" x14ac:dyDescent="0.25">
@@ -10111,7 +10111,7 @@
         <v>10</v>
       </c>
       <c r="F328">
-        <v>837</v>
+        <v>842</v>
       </c>
     </row>
     <row r="329" spans="1:6" x14ac:dyDescent="0.25">
@@ -10131,7 +10131,7 @@
         <v>10</v>
       </c>
       <c r="F329">
-        <v>494</v>
+        <v>355</v>
       </c>
     </row>
     <row r="330" spans="1:6" x14ac:dyDescent="0.25">
@@ -10151,7 +10151,7 @@
         <v>10</v>
       </c>
       <c r="F330">
-        <v>708</v>
+        <v>238</v>
       </c>
     </row>
     <row r="331" spans="1:6" x14ac:dyDescent="0.25">
@@ -10171,7 +10171,7 @@
         <v>10</v>
       </c>
       <c r="F331">
-        <v>480</v>
+        <v>777</v>
       </c>
     </row>
     <row r="332" spans="1:6" x14ac:dyDescent="0.25">
@@ -10191,7 +10191,7 @@
         <v>10</v>
       </c>
       <c r="F332">
-        <v>289</v>
+        <v>383</v>
       </c>
     </row>
     <row r="333" spans="1:6" x14ac:dyDescent="0.25">
@@ -10211,7 +10211,7 @@
         <v>10</v>
       </c>
       <c r="F333">
-        <v>971</v>
+        <v>479</v>
       </c>
     </row>
     <row r="334" spans="1:6" x14ac:dyDescent="0.25">
@@ -10231,7 +10231,7 @@
         <v>10</v>
       </c>
       <c r="F334">
-        <v>940</v>
+        <v>392</v>
       </c>
     </row>
     <row r="335" spans="1:6" x14ac:dyDescent="0.25">
@@ -10251,7 +10251,7 @@
         <v>10</v>
       </c>
       <c r="F335">
-        <v>500</v>
+        <v>969</v>
       </c>
     </row>
     <row r="336" spans="1:6" x14ac:dyDescent="0.25">
@@ -10271,7 +10271,7 @@
         <v>10</v>
       </c>
       <c r="F336">
-        <v>666</v>
+        <v>211</v>
       </c>
     </row>
     <row r="337" spans="1:6" x14ac:dyDescent="0.25">
@@ -10291,7 +10291,7 @@
         <v>10</v>
       </c>
       <c r="F337">
-        <v>200</v>
+        <v>948</v>
       </c>
     </row>
     <row r="338" spans="1:6" x14ac:dyDescent="0.25">
@@ -10311,7 +10311,7 @@
         <v>10</v>
       </c>
       <c r="F338">
-        <v>896</v>
+        <v>341</v>
       </c>
     </row>
     <row r="339" spans="1:6" x14ac:dyDescent="0.25">
@@ -10331,7 +10331,7 @@
         <v>10</v>
       </c>
       <c r="F339">
-        <v>976</v>
+        <v>612</v>
       </c>
     </row>
     <row r="340" spans="1:6" x14ac:dyDescent="0.25">
@@ -10351,7 +10351,7 @@
         <v>10</v>
       </c>
       <c r="F340">
-        <v>748</v>
+        <v>616</v>
       </c>
     </row>
     <row r="341" spans="1:6" x14ac:dyDescent="0.25">
@@ -10371,7 +10371,7 @@
         <v>10</v>
       </c>
       <c r="F341">
-        <v>230</v>
+        <v>810</v>
       </c>
     </row>
     <row r="342" spans="1:6" x14ac:dyDescent="0.25">
@@ -10391,7 +10391,7 @@
         <v>10</v>
       </c>
       <c r="F342">
-        <v>353</v>
+        <v>701</v>
       </c>
     </row>
     <row r="343" spans="1:6" x14ac:dyDescent="0.25">
@@ -10411,7 +10411,7 @@
         <v>10</v>
       </c>
       <c r="F343">
-        <v>550</v>
+        <v>809</v>
       </c>
     </row>
     <row r="344" spans="1:6" x14ac:dyDescent="0.25">
@@ -10431,7 +10431,7 @@
         <v>10</v>
       </c>
       <c r="F344">
-        <v>622</v>
+        <v>968</v>
       </c>
     </row>
     <row r="345" spans="1:6" x14ac:dyDescent="0.25">
@@ -10451,7 +10451,7 @@
         <v>10</v>
       </c>
       <c r="F345">
-        <v>953</v>
+        <v>539</v>
       </c>
     </row>
     <row r="346" spans="1:6" x14ac:dyDescent="0.25">
@@ -10471,7 +10471,7 @@
         <v>10</v>
       </c>
       <c r="F346">
-        <v>820</v>
+        <v>748</v>
       </c>
     </row>
     <row r="347" spans="1:6" x14ac:dyDescent="0.25">
@@ -10491,7 +10491,7 @@
         <v>10</v>
       </c>
       <c r="F347">
-        <v>922</v>
+        <v>365</v>
       </c>
     </row>
     <row r="348" spans="1:6" x14ac:dyDescent="0.25">
@@ -10511,7 +10511,7 @@
         <v>10</v>
       </c>
       <c r="F348">
-        <v>756</v>
+        <v>857</v>
       </c>
     </row>
     <row r="349" spans="1:6" x14ac:dyDescent="0.25">
@@ -10531,7 +10531,7 @@
         <v>10</v>
       </c>
       <c r="F349">
-        <v>464</v>
+        <v>346</v>
       </c>
     </row>
     <row r="350" spans="1:6" x14ac:dyDescent="0.25">
@@ -10551,7 +10551,7 @@
         <v>10</v>
       </c>
       <c r="F350">
-        <v>612</v>
+        <v>790</v>
       </c>
     </row>
     <row r="351" spans="1:6" x14ac:dyDescent="0.25">
@@ -10571,7 +10571,7 @@
         <v>10</v>
       </c>
       <c r="F351">
-        <v>813</v>
+        <v>693</v>
       </c>
     </row>
     <row r="352" spans="1:6" x14ac:dyDescent="0.25">
@@ -10591,7 +10591,7 @@
         <v>10</v>
       </c>
       <c r="F352">
-        <v>264</v>
+        <v>951</v>
       </c>
     </row>
     <row r="353" spans="1:6" x14ac:dyDescent="0.25">
@@ -10611,7 +10611,7 @@
         <v>10</v>
       </c>
       <c r="F353">
-        <v>371</v>
+        <v>242</v>
       </c>
     </row>
     <row r="354" spans="1:6" x14ac:dyDescent="0.25">
@@ -10631,7 +10631,7 @@
         <v>10</v>
       </c>
       <c r="F354">
-        <v>655</v>
+        <v>932</v>
       </c>
     </row>
     <row r="355" spans="1:6" x14ac:dyDescent="0.25">
@@ -10651,7 +10651,7 @@
         <v>10</v>
       </c>
       <c r="F355">
-        <v>811</v>
+        <v>952</v>
       </c>
     </row>
     <row r="356" spans="1:6" x14ac:dyDescent="0.25">
@@ -10671,7 +10671,7 @@
         <v>10</v>
       </c>
       <c r="F356">
-        <v>391</v>
+        <v>648</v>
       </c>
     </row>
     <row r="357" spans="1:6" x14ac:dyDescent="0.25">
@@ -10691,7 +10691,7 @@
         <v>10</v>
       </c>
       <c r="F357">
-        <v>222</v>
+        <v>402</v>
       </c>
     </row>
     <row r="358" spans="1:6" x14ac:dyDescent="0.25">
@@ -10711,7 +10711,7 @@
         <v>10</v>
       </c>
       <c r="F358">
-        <v>955</v>
+        <v>504</v>
       </c>
     </row>
     <row r="359" spans="1:6" x14ac:dyDescent="0.25">
@@ -10731,7 +10731,7 @@
         <v>10</v>
       </c>
       <c r="F359">
-        <v>738</v>
+        <v>973</v>
       </c>
     </row>
     <row r="360" spans="1:6" x14ac:dyDescent="0.25">
@@ -10751,7 +10751,7 @@
         <v>10</v>
       </c>
       <c r="F360">
-        <v>960</v>
+        <v>581</v>
       </c>
     </row>
     <row r="361" spans="1:6" x14ac:dyDescent="0.25">
@@ -10771,7 +10771,7 @@
         <v>10</v>
       </c>
       <c r="F361">
-        <v>754</v>
+        <v>762</v>
       </c>
     </row>
     <row r="362" spans="1:6" x14ac:dyDescent="0.25">
@@ -10791,7 +10791,7 @@
         <v>10</v>
       </c>
       <c r="F362">
-        <v>640</v>
+        <v>956</v>
       </c>
     </row>
     <row r="363" spans="1:6" x14ac:dyDescent="0.25">
@@ -10811,7 +10811,7 @@
         <v>10</v>
       </c>
       <c r="F363">
-        <v>871</v>
+        <v>337</v>
       </c>
     </row>
     <row r="364" spans="1:6" x14ac:dyDescent="0.25">
@@ -10831,7 +10831,7 @@
         <v>10</v>
       </c>
       <c r="F364">
-        <v>757</v>
+        <v>839</v>
       </c>
     </row>
     <row r="365" spans="1:6" x14ac:dyDescent="0.25">
@@ -10851,7 +10851,7 @@
         <v>10</v>
       </c>
       <c r="F365">
-        <v>520</v>
+        <v>672</v>
       </c>
     </row>
     <row r="366" spans="1:6" x14ac:dyDescent="0.25">
@@ -10871,7 +10871,7 @@
         <v>10</v>
       </c>
       <c r="F366">
-        <v>602</v>
+        <v>554</v>
       </c>
     </row>
     <row r="367" spans="1:6" x14ac:dyDescent="0.25">
@@ -10891,7 +10891,7 @@
         <v>10</v>
       </c>
       <c r="F367">
-        <v>951</v>
+        <v>520</v>
       </c>
     </row>
     <row r="368" spans="1:6" x14ac:dyDescent="0.25">
@@ -10911,7 +10911,7 @@
         <v>10</v>
       </c>
       <c r="F368">
-        <v>501</v>
+        <v>675</v>
       </c>
     </row>
     <row r="369" spans="1:6" x14ac:dyDescent="0.25">
@@ -10931,7 +10931,7 @@
         <v>10</v>
       </c>
       <c r="F369">
-        <v>302</v>
+        <v>920</v>
       </c>
     </row>
     <row r="370" spans="1:6" x14ac:dyDescent="0.25">
@@ -10951,7 +10951,7 @@
         <v>10</v>
       </c>
       <c r="F370">
-        <v>829</v>
+        <v>615</v>
       </c>
     </row>
     <row r="371" spans="1:6" x14ac:dyDescent="0.25">
@@ -10971,7 +10971,7 @@
         <v>10</v>
       </c>
       <c r="F371">
-        <v>423</v>
+        <v>517</v>
       </c>
     </row>
     <row r="372" spans="1:6" x14ac:dyDescent="0.25">
@@ -10991,7 +10991,7 @@
         <v>10</v>
       </c>
       <c r="F372">
-        <v>333</v>
+        <v>568</v>
       </c>
     </row>
     <row r="373" spans="1:6" x14ac:dyDescent="0.25">
@@ -11011,7 +11011,7 @@
         <v>10</v>
       </c>
       <c r="F373">
-        <v>994</v>
+        <v>997</v>
       </c>
     </row>
     <row r="374" spans="1:6" x14ac:dyDescent="0.25">
@@ -11031,7 +11031,7 @@
         <v>10</v>
       </c>
       <c r="F374">
-        <v>981</v>
+        <v>768</v>
       </c>
     </row>
     <row r="375" spans="1:6" x14ac:dyDescent="0.25">
@@ -11051,7 +11051,7 @@
         <v>10</v>
       </c>
       <c r="F375">
-        <v>976</v>
+        <v>386</v>
       </c>
     </row>
     <row r="376" spans="1:6" x14ac:dyDescent="0.25">
@@ -11071,7 +11071,7 @@
         <v>10</v>
       </c>
       <c r="F376">
-        <v>334</v>
+        <v>522</v>
       </c>
     </row>
     <row r="377" spans="1:6" x14ac:dyDescent="0.25">
@@ -11091,7 +11091,7 @@
         <v>10</v>
       </c>
       <c r="F377">
-        <v>268</v>
+        <v>556</v>
       </c>
     </row>
     <row r="378" spans="1:6" x14ac:dyDescent="0.25">
@@ -11111,7 +11111,7 @@
         <v>10</v>
       </c>
       <c r="F378">
-        <v>786</v>
+        <v>750</v>
       </c>
     </row>
     <row r="379" spans="1:6" x14ac:dyDescent="0.25">
@@ -11131,7 +11131,7 @@
         <v>10</v>
       </c>
       <c r="F379">
-        <v>663</v>
+        <v>357</v>
       </c>
     </row>
     <row r="380" spans="1:6" x14ac:dyDescent="0.25">
@@ -11151,7 +11151,7 @@
         <v>10</v>
       </c>
       <c r="F380">
-        <v>251</v>
+        <v>898</v>
       </c>
     </row>
     <row r="381" spans="1:6" x14ac:dyDescent="0.25">
@@ -11171,7 +11171,7 @@
         <v>10</v>
       </c>
       <c r="F381">
-        <v>756</v>
+        <v>559</v>
       </c>
     </row>
     <row r="382" spans="1:6" x14ac:dyDescent="0.25">
@@ -11191,7 +11191,7 @@
         <v>10</v>
       </c>
       <c r="F382">
-        <v>826</v>
+        <v>238</v>
       </c>
     </row>
     <row r="383" spans="1:6" x14ac:dyDescent="0.25">
@@ -11211,7 +11211,7 @@
         <v>10</v>
       </c>
       <c r="F383">
-        <v>736</v>
+        <v>623</v>
       </c>
     </row>
     <row r="384" spans="1:6" x14ac:dyDescent="0.25">
@@ -11231,7 +11231,7 @@
         <v>10</v>
       </c>
       <c r="F384">
-        <v>322</v>
+        <v>585</v>
       </c>
     </row>
     <row r="385" spans="1:6" x14ac:dyDescent="0.25">
@@ -11251,7 +11251,7 @@
         <v>10</v>
       </c>
       <c r="F385">
-        <v>684</v>
+        <v>315</v>
       </c>
     </row>
     <row r="386" spans="1:6" x14ac:dyDescent="0.25">
@@ -11271,7 +11271,7 @@
         <v>10</v>
       </c>
       <c r="F386">
-        <v>423</v>
+        <v>904</v>
       </c>
     </row>
     <row r="387" spans="1:6" x14ac:dyDescent="0.25">
@@ -11291,7 +11291,7 @@
         <v>10</v>
       </c>
       <c r="F387">
-        <v>200</v>
+        <v>408</v>
       </c>
     </row>
     <row r="388" spans="1:6" x14ac:dyDescent="0.25">
@@ -11311,7 +11311,7 @@
         <v>10</v>
       </c>
       <c r="F388">
-        <v>411</v>
+        <v>483</v>
       </c>
     </row>
     <row r="389" spans="1:6" x14ac:dyDescent="0.25">
@@ -11331,7 +11331,7 @@
         <v>10</v>
       </c>
       <c r="F389">
-        <v>388</v>
+        <v>488</v>
       </c>
     </row>
     <row r="390" spans="1:6" x14ac:dyDescent="0.25">
@@ -11351,7 +11351,7 @@
         <v>10</v>
       </c>
       <c r="F390">
-        <v>601</v>
+        <v>996</v>
       </c>
     </row>
     <row r="391" spans="1:6" x14ac:dyDescent="0.25">
@@ -11371,7 +11371,7 @@
         <v>10</v>
       </c>
       <c r="F391">
-        <v>836</v>
+        <v>482</v>
       </c>
     </row>
     <row r="392" spans="1:6" x14ac:dyDescent="0.25">
@@ -11391,7 +11391,7 @@
         <v>10</v>
       </c>
       <c r="F392">
-        <v>798</v>
+        <v>879</v>
       </c>
     </row>
     <row r="393" spans="1:6" x14ac:dyDescent="0.25">
@@ -11411,7 +11411,7 @@
         <v>10</v>
       </c>
       <c r="F393">
-        <v>656</v>
+        <v>983</v>
       </c>
     </row>
     <row r="394" spans="1:6" x14ac:dyDescent="0.25">
@@ -11431,7 +11431,7 @@
         <v>10</v>
       </c>
       <c r="F394">
-        <v>676</v>
+        <v>265</v>
       </c>
     </row>
     <row r="395" spans="1:6" x14ac:dyDescent="0.25">
@@ -11451,7 +11451,7 @@
         <v>10</v>
       </c>
       <c r="F395">
-        <v>319</v>
+        <v>245</v>
       </c>
     </row>
     <row r="396" spans="1:6" x14ac:dyDescent="0.25">
@@ -11471,7 +11471,7 @@
         <v>10</v>
       </c>
       <c r="F396">
-        <v>811</v>
+        <v>268</v>
       </c>
     </row>
     <row r="397" spans="1:6" x14ac:dyDescent="0.25">
@@ -11511,7 +11511,7 @@
         <v>10</v>
       </c>
       <c r="F398">
-        <v>221</v>
+        <v>518</v>
       </c>
     </row>
     <row r="399" spans="1:6" x14ac:dyDescent="0.25">
@@ -11531,7 +11531,7 @@
         <v>10</v>
       </c>
       <c r="F399">
-        <v>979</v>
+        <v>275</v>
       </c>
     </row>
     <row r="400" spans="1:6" x14ac:dyDescent="0.25">
@@ -11551,7 +11551,7 @@
         <v>10</v>
       </c>
       <c r="F400">
-        <v>845</v>
+        <v>327</v>
       </c>
     </row>
     <row r="401" spans="1:6" x14ac:dyDescent="0.25">
@@ -11571,7 +11571,7 @@
         <v>10</v>
       </c>
       <c r="F401">
-        <v>782</v>
+        <v>308</v>
       </c>
     </row>
     <row r="402" spans="1:6" x14ac:dyDescent="0.25">
@@ -11591,7 +11591,7 @@
         <v>10</v>
       </c>
       <c r="F402">
-        <v>406</v>
+        <v>387</v>
       </c>
     </row>
     <row r="403" spans="1:6" x14ac:dyDescent="0.25">
@@ -11611,7 +11611,7 @@
         <v>10</v>
       </c>
       <c r="F403">
-        <v>758</v>
+        <v>251</v>
       </c>
     </row>
     <row r="404" spans="1:6" x14ac:dyDescent="0.25">
@@ -11631,7 +11631,7 @@
         <v>10</v>
       </c>
       <c r="F404">
-        <v>837</v>
+        <v>264</v>
       </c>
     </row>
     <row r="405" spans="1:6" x14ac:dyDescent="0.25">
@@ -11651,7 +11651,7 @@
         <v>10</v>
       </c>
       <c r="F405">
-        <v>815</v>
+        <v>503</v>
       </c>
     </row>
     <row r="406" spans="1:6" x14ac:dyDescent="0.25">
@@ -11671,7 +11671,7 @@
         <v>10</v>
       </c>
       <c r="F406">
-        <v>639</v>
+        <v>910</v>
       </c>
     </row>
     <row r="407" spans="1:6" x14ac:dyDescent="0.25">
@@ -11691,7 +11691,7 @@
         <v>10</v>
       </c>
       <c r="F407">
-        <v>291</v>
+        <v>878</v>
       </c>
     </row>
     <row r="408" spans="1:6" x14ac:dyDescent="0.25">
@@ -11711,7 +11711,7 @@
         <v>10</v>
       </c>
       <c r="F408">
-        <v>228</v>
+        <v>538</v>
       </c>
     </row>
     <row r="409" spans="1:6" x14ac:dyDescent="0.25">
@@ -11731,7 +11731,7 @@
         <v>10</v>
       </c>
       <c r="F409">
-        <v>220</v>
+        <v>731</v>
       </c>
     </row>
     <row r="410" spans="1:6" x14ac:dyDescent="0.25">
@@ -11751,7 +11751,7 @@
         <v>10</v>
       </c>
       <c r="F410">
-        <v>715</v>
+        <v>837</v>
       </c>
     </row>
     <row r="411" spans="1:6" x14ac:dyDescent="0.25">
@@ -11771,7 +11771,7 @@
         <v>10</v>
       </c>
       <c r="F411">
-        <v>838</v>
+        <v>980</v>
       </c>
     </row>
     <row r="412" spans="1:6" x14ac:dyDescent="0.25">
@@ -11791,7 +11791,7 @@
         <v>10</v>
       </c>
       <c r="F412">
-        <v>417</v>
+        <v>499</v>
       </c>
     </row>
     <row r="413" spans="1:6" x14ac:dyDescent="0.25">
@@ -11811,7 +11811,7 @@
         <v>10</v>
       </c>
       <c r="F413">
-        <v>605</v>
+        <v>697</v>
       </c>
     </row>
     <row r="414" spans="1:6" x14ac:dyDescent="0.25">
@@ -11831,7 +11831,7 @@
         <v>10</v>
       </c>
       <c r="F414">
-        <v>390</v>
+        <v>475</v>
       </c>
     </row>
     <row r="415" spans="1:6" x14ac:dyDescent="0.25">
@@ -11851,7 +11851,7 @@
         <v>10</v>
       </c>
       <c r="F415">
-        <v>213</v>
+        <v>717</v>
       </c>
     </row>
     <row r="416" spans="1:6" x14ac:dyDescent="0.25">
@@ -11871,7 +11871,7 @@
         <v>10</v>
       </c>
       <c r="F416">
-        <v>409</v>
+        <v>994</v>
       </c>
     </row>
     <row r="417" spans="1:6" x14ac:dyDescent="0.25">
@@ -11891,7 +11891,7 @@
         <v>10</v>
       </c>
       <c r="F417">
-        <v>397</v>
+        <v>534</v>
       </c>
     </row>
     <row r="418" spans="1:6" x14ac:dyDescent="0.25">
@@ -11911,7 +11911,7 @@
         <v>10</v>
       </c>
       <c r="F418">
-        <v>319</v>
+        <v>362</v>
       </c>
     </row>
     <row r="419" spans="1:6" x14ac:dyDescent="0.25">
@@ -11931,7 +11931,7 @@
         <v>10</v>
       </c>
       <c r="F419">
-        <v>315</v>
+        <v>780</v>
       </c>
     </row>
     <row r="420" spans="1:6" x14ac:dyDescent="0.25">
@@ -11951,7 +11951,7 @@
         <v>10</v>
       </c>
       <c r="F420">
-        <v>257</v>
+        <v>369</v>
       </c>
     </row>
     <row r="421" spans="1:6" x14ac:dyDescent="0.25">
@@ -11971,7 +11971,7 @@
         <v>10</v>
       </c>
       <c r="F421">
-        <v>584</v>
+        <v>646</v>
       </c>
     </row>
     <row r="422" spans="1:6" x14ac:dyDescent="0.25">
@@ -11991,7 +11991,7 @@
         <v>10</v>
       </c>
       <c r="F422">
-        <v>305</v>
+        <v>295</v>
       </c>
     </row>
     <row r="423" spans="1:6" x14ac:dyDescent="0.25">
@@ -12011,7 +12011,7 @@
         <v>10</v>
       </c>
       <c r="F423">
-        <v>202</v>
+        <v>285</v>
       </c>
     </row>
     <row r="424" spans="1:6" x14ac:dyDescent="0.25">
@@ -12031,7 +12031,7 @@
         <v>10</v>
       </c>
       <c r="F424">
-        <v>982</v>
+        <v>986</v>
       </c>
     </row>
     <row r="425" spans="1:6" x14ac:dyDescent="0.25">
@@ -12051,7 +12051,7 @@
         <v>10</v>
       </c>
       <c r="F425">
-        <v>569</v>
+        <v>377</v>
       </c>
     </row>
     <row r="426" spans="1:6" x14ac:dyDescent="0.25">
@@ -12071,7 +12071,7 @@
         <v>10</v>
       </c>
       <c r="F426">
-        <v>685</v>
+        <v>837</v>
       </c>
     </row>
     <row r="427" spans="1:6" x14ac:dyDescent="0.25">
@@ -12091,7 +12091,7 @@
         <v>10</v>
       </c>
       <c r="F427">
-        <v>773</v>
+        <v>508</v>
       </c>
     </row>
     <row r="428" spans="1:6" x14ac:dyDescent="0.25">
@@ -12111,7 +12111,7 @@
         <v>10</v>
       </c>
       <c r="F428">
-        <v>759</v>
+        <v>744</v>
       </c>
     </row>
     <row r="429" spans="1:6" x14ac:dyDescent="0.25">
@@ -12131,7 +12131,7 @@
         <v>10</v>
       </c>
       <c r="F429">
-        <v>221</v>
+        <v>852</v>
       </c>
     </row>
     <row r="430" spans="1:6" x14ac:dyDescent="0.25">
@@ -12151,7 +12151,7 @@
         <v>10</v>
       </c>
       <c r="F430">
-        <v>752</v>
+        <v>781</v>
       </c>
     </row>
     <row r="431" spans="1:6" x14ac:dyDescent="0.25">
@@ -12171,7 +12171,7 @@
         <v>10</v>
       </c>
       <c r="F431">
-        <v>918</v>
+        <v>593</v>
       </c>
     </row>
     <row r="432" spans="1:6" x14ac:dyDescent="0.25">
@@ -12191,7 +12191,7 @@
         <v>10</v>
       </c>
       <c r="F432">
-        <v>520</v>
+        <v>685</v>
       </c>
     </row>
     <row r="433" spans="1:6" x14ac:dyDescent="0.25">
@@ -12211,7 +12211,7 @@
         <v>10</v>
       </c>
       <c r="F433">
-        <v>593</v>
+        <v>294</v>
       </c>
     </row>
     <row r="434" spans="1:6" x14ac:dyDescent="0.25">
@@ -12231,7 +12231,7 @@
         <v>10</v>
       </c>
       <c r="F434">
-        <v>751</v>
+        <v>943</v>
       </c>
     </row>
     <row r="435" spans="1:6" x14ac:dyDescent="0.25">
@@ -12251,7 +12251,7 @@
         <v>10</v>
       </c>
       <c r="F435">
-        <v>318</v>
+        <v>383</v>
       </c>
     </row>
     <row r="436" spans="1:6" x14ac:dyDescent="0.25">
@@ -12271,7 +12271,7 @@
         <v>10</v>
       </c>
       <c r="F436">
-        <v>858</v>
+        <v>246</v>
       </c>
     </row>
     <row r="437" spans="1:6" x14ac:dyDescent="0.25">
@@ -12291,7 +12291,7 @@
         <v>10</v>
       </c>
       <c r="F437">
-        <v>551</v>
+        <v>610</v>
       </c>
     </row>
     <row r="438" spans="1:6" x14ac:dyDescent="0.25">
@@ -12311,7 +12311,7 @@
         <v>10</v>
       </c>
       <c r="F438">
-        <v>931</v>
+        <v>730</v>
       </c>
     </row>
     <row r="439" spans="1:6" x14ac:dyDescent="0.25">
@@ -12331,7 +12331,7 @@
         <v>10</v>
       </c>
       <c r="F439">
-        <v>323</v>
+        <v>433</v>
       </c>
     </row>
     <row r="440" spans="1:6" x14ac:dyDescent="0.25">
@@ -12351,7 +12351,7 @@
         <v>10</v>
       </c>
       <c r="F440">
-        <v>815</v>
+        <v>380</v>
       </c>
     </row>
     <row r="441" spans="1:6" x14ac:dyDescent="0.25">
@@ -12371,7 +12371,7 @@
         <v>10</v>
       </c>
       <c r="F441">
-        <v>347</v>
+        <v>448</v>
       </c>
     </row>
     <row r="442" spans="1:6" x14ac:dyDescent="0.25">
@@ -12391,7 +12391,7 @@
         <v>10</v>
       </c>
       <c r="F442">
-        <v>767</v>
+        <v>591</v>
       </c>
     </row>
     <row r="443" spans="1:6" x14ac:dyDescent="0.25">
@@ -12411,7 +12411,7 @@
         <v>10</v>
       </c>
       <c r="F443">
-        <v>846</v>
+        <v>527</v>
       </c>
     </row>
     <row r="444" spans="1:6" x14ac:dyDescent="0.25">
@@ -12431,7 +12431,7 @@
         <v>10</v>
       </c>
       <c r="F444">
-        <v>772</v>
+        <v>225</v>
       </c>
     </row>
     <row r="445" spans="1:6" x14ac:dyDescent="0.25">
@@ -12451,7 +12451,7 @@
         <v>10</v>
       </c>
       <c r="F445">
-        <v>991</v>
+        <v>527</v>
       </c>
     </row>
     <row r="446" spans="1:6" x14ac:dyDescent="0.25">
@@ -12471,7 +12471,7 @@
         <v>10</v>
       </c>
       <c r="F446">
-        <v>243</v>
+        <v>356</v>
       </c>
     </row>
     <row r="447" spans="1:6" x14ac:dyDescent="0.25">
@@ -12491,7 +12491,7 @@
         <v>10</v>
       </c>
       <c r="F447">
-        <v>694</v>
+        <v>472</v>
       </c>
     </row>
     <row r="448" spans="1:6" x14ac:dyDescent="0.25">
@@ -12511,7 +12511,7 @@
         <v>10</v>
       </c>
       <c r="F448">
-        <v>963</v>
+        <v>428</v>
       </c>
     </row>
     <row r="449" spans="1:6" x14ac:dyDescent="0.25">
@@ -12531,7 +12531,7 @@
         <v>10</v>
       </c>
       <c r="F449">
-        <v>855</v>
+        <v>840</v>
       </c>
     </row>
     <row r="450" spans="1:6" x14ac:dyDescent="0.25">
@@ -12551,7 +12551,7 @@
         <v>10</v>
       </c>
       <c r="F450">
-        <v>554</v>
+        <v>834</v>
       </c>
     </row>
     <row r="451" spans="1:6" x14ac:dyDescent="0.25">
@@ -12571,7 +12571,7 @@
         <v>10</v>
       </c>
       <c r="F451">
-        <v>317</v>
+        <v>512</v>
       </c>
     </row>
     <row r="452" spans="1:6" x14ac:dyDescent="0.25">
@@ -12591,7 +12591,7 @@
         <v>10</v>
       </c>
       <c r="F452">
-        <v>947</v>
+        <v>624</v>
       </c>
     </row>
     <row r="453" spans="1:6" x14ac:dyDescent="0.25">
@@ -12611,7 +12611,7 @@
         <v>10</v>
       </c>
       <c r="F453">
-        <v>642</v>
+        <v>531</v>
       </c>
     </row>
     <row r="454" spans="1:6" x14ac:dyDescent="0.25">
@@ -12631,7 +12631,7 @@
         <v>10</v>
       </c>
       <c r="F454">
-        <v>378</v>
+        <v>666</v>
       </c>
     </row>
     <row r="455" spans="1:6" x14ac:dyDescent="0.25">
@@ -12651,7 +12651,7 @@
         <v>10</v>
       </c>
       <c r="F455">
-        <v>712</v>
+        <v>877</v>
       </c>
     </row>
     <row r="456" spans="1:6" x14ac:dyDescent="0.25">
@@ -12671,7 +12671,7 @@
         <v>10</v>
       </c>
       <c r="F456">
-        <v>421</v>
+        <v>960</v>
       </c>
     </row>
     <row r="457" spans="1:6" x14ac:dyDescent="0.25">
@@ -12691,7 +12691,7 @@
         <v>10</v>
       </c>
       <c r="F457">
-        <v>580</v>
+        <v>952</v>
       </c>
     </row>
     <row r="458" spans="1:6" x14ac:dyDescent="0.25">
@@ -12711,7 +12711,7 @@
         <v>10</v>
       </c>
       <c r="F458">
-        <v>956</v>
+        <v>465</v>
       </c>
     </row>
     <row r="459" spans="1:6" x14ac:dyDescent="0.25">
@@ -12731,7 +12731,7 @@
         <v>10</v>
       </c>
       <c r="F459">
-        <v>980</v>
+        <v>438</v>
       </c>
     </row>
     <row r="460" spans="1:6" x14ac:dyDescent="0.25">
@@ -12751,7 +12751,7 @@
         <v>10</v>
       </c>
       <c r="F460">
-        <v>505</v>
+        <v>290</v>
       </c>
     </row>
     <row r="461" spans="1:6" x14ac:dyDescent="0.25">
@@ -12771,7 +12771,7 @@
         <v>10</v>
       </c>
       <c r="F461">
-        <v>905</v>
+        <v>921</v>
       </c>
     </row>
     <row r="462" spans="1:6" x14ac:dyDescent="0.25">
@@ -12791,7 +12791,7 @@
         <v>10</v>
       </c>
       <c r="F462">
-        <v>670</v>
+        <v>535</v>
       </c>
     </row>
     <row r="463" spans="1:6" x14ac:dyDescent="0.25">
@@ -12811,7 +12811,7 @@
         <v>10</v>
       </c>
       <c r="F463">
-        <v>562</v>
+        <v>600</v>
       </c>
     </row>
     <row r="464" spans="1:6" x14ac:dyDescent="0.25">
@@ -12831,7 +12831,7 @@
         <v>10</v>
       </c>
       <c r="F464">
-        <v>967</v>
+        <v>525</v>
       </c>
     </row>
     <row r="465" spans="1:6" x14ac:dyDescent="0.25">
@@ -12851,7 +12851,7 @@
         <v>10</v>
       </c>
       <c r="F465">
-        <v>439</v>
+        <v>344</v>
       </c>
     </row>
     <row r="466" spans="1:6" x14ac:dyDescent="0.25">
@@ -12871,7 +12871,7 @@
         <v>10</v>
       </c>
       <c r="F466">
-        <v>596</v>
+        <v>366</v>
       </c>
     </row>
     <row r="467" spans="1:6" x14ac:dyDescent="0.25">
@@ -12891,7 +12891,7 @@
         <v>10</v>
       </c>
       <c r="F467">
-        <v>350</v>
+        <v>251</v>
       </c>
     </row>
     <row r="468" spans="1:6" x14ac:dyDescent="0.25">
@@ -12911,7 +12911,7 @@
         <v>10</v>
       </c>
       <c r="F468">
-        <v>962</v>
+        <v>973</v>
       </c>
     </row>
     <row r="469" spans="1:6" x14ac:dyDescent="0.25">
@@ -12931,7 +12931,7 @@
         <v>10</v>
       </c>
       <c r="F469">
-        <v>688</v>
+        <v>616</v>
       </c>
     </row>
     <row r="470" spans="1:6" x14ac:dyDescent="0.25">
@@ -12951,7 +12951,7 @@
         <v>10</v>
       </c>
       <c r="F470">
-        <v>247</v>
+        <v>216</v>
       </c>
     </row>
     <row r="471" spans="1:6" x14ac:dyDescent="0.25">
@@ -12971,7 +12971,7 @@
         <v>10</v>
       </c>
       <c r="F471">
-        <v>698</v>
+        <v>326</v>
       </c>
     </row>
     <row r="472" spans="1:6" x14ac:dyDescent="0.25">
@@ -12991,7 +12991,7 @@
         <v>10</v>
       </c>
       <c r="F472">
-        <v>988</v>
+        <v>634</v>
       </c>
     </row>
     <row r="473" spans="1:6" x14ac:dyDescent="0.25">
@@ -13011,7 +13011,7 @@
         <v>10</v>
       </c>
       <c r="F473">
-        <v>525</v>
+        <v>608</v>
       </c>
     </row>
     <row r="474" spans="1:6" x14ac:dyDescent="0.25">
@@ -13031,7 +13031,7 @@
         <v>10</v>
       </c>
       <c r="F474">
-        <v>694</v>
+        <v>832</v>
       </c>
     </row>
     <row r="475" spans="1:6" x14ac:dyDescent="0.25">
@@ -13051,7 +13051,7 @@
         <v>10</v>
       </c>
       <c r="F475">
-        <v>626</v>
+        <v>663</v>
       </c>
     </row>
     <row r="476" spans="1:6" x14ac:dyDescent="0.25">
@@ -13071,7 +13071,7 @@
         <v>10</v>
       </c>
       <c r="F476">
-        <v>241</v>
+        <v>757</v>
       </c>
     </row>
     <row r="477" spans="1:6" x14ac:dyDescent="0.25">
@@ -13091,7 +13091,7 @@
         <v>10</v>
       </c>
       <c r="F477">
-        <v>689</v>
+        <v>961</v>
       </c>
     </row>
     <row r="478" spans="1:6" x14ac:dyDescent="0.25">
@@ -13111,7 +13111,7 @@
         <v>10</v>
       </c>
       <c r="F478">
-        <v>425</v>
+        <v>924</v>
       </c>
     </row>
     <row r="479" spans="1:6" x14ac:dyDescent="0.25">
@@ -13131,7 +13131,7 @@
         <v>10</v>
       </c>
       <c r="F479">
-        <v>568</v>
+        <v>210</v>
       </c>
     </row>
     <row r="480" spans="1:6" x14ac:dyDescent="0.25">
@@ -13151,7 +13151,7 @@
         <v>10</v>
       </c>
       <c r="F480">
-        <v>808</v>
+        <v>646</v>
       </c>
     </row>
     <row r="481" spans="1:6" x14ac:dyDescent="0.25">
@@ -13171,7 +13171,7 @@
         <v>10</v>
       </c>
       <c r="F481">
-        <v>920</v>
+        <v>894</v>
       </c>
     </row>
     <row r="482" spans="1:6" x14ac:dyDescent="0.25">
@@ -13191,7 +13191,7 @@
         <v>10</v>
       </c>
       <c r="F482">
-        <v>511</v>
+        <v>201</v>
       </c>
     </row>
     <row r="483" spans="1:6" x14ac:dyDescent="0.25">
@@ -13211,7 +13211,7 @@
         <v>10</v>
       </c>
       <c r="F483">
-        <v>276</v>
+        <v>311</v>
       </c>
     </row>
     <row r="484" spans="1:6" x14ac:dyDescent="0.25">
@@ -13231,7 +13231,7 @@
         <v>10</v>
       </c>
       <c r="F484">
-        <v>407</v>
+        <v>566</v>
       </c>
     </row>
     <row r="485" spans="1:6" x14ac:dyDescent="0.25">
@@ -13251,7 +13251,7 @@
         <v>10</v>
       </c>
       <c r="F485">
-        <v>568</v>
+        <v>825</v>
       </c>
     </row>
     <row r="486" spans="1:6" x14ac:dyDescent="0.25">
@@ -13271,7 +13271,7 @@
         <v>10</v>
       </c>
       <c r="F486">
-        <v>926</v>
+        <v>971</v>
       </c>
     </row>
     <row r="487" spans="1:6" x14ac:dyDescent="0.25">
@@ -13291,7 +13291,7 @@
         <v>10</v>
       </c>
       <c r="F487">
-        <v>403</v>
+        <v>461</v>
       </c>
     </row>
     <row r="488" spans="1:6" x14ac:dyDescent="0.25">
@@ -13311,7 +13311,7 @@
         <v>10</v>
       </c>
       <c r="F488">
-        <v>885</v>
+        <v>211</v>
       </c>
     </row>
     <row r="489" spans="1:6" x14ac:dyDescent="0.25">
@@ -13331,7 +13331,7 @@
         <v>10</v>
       </c>
       <c r="F489">
-        <v>894</v>
+        <v>546</v>
       </c>
     </row>
     <row r="490" spans="1:6" x14ac:dyDescent="0.25">
@@ -13351,7 +13351,7 @@
         <v>10</v>
       </c>
       <c r="F490">
-        <v>633</v>
+        <v>690</v>
       </c>
     </row>
     <row r="491" spans="1:6" x14ac:dyDescent="0.25">
@@ -13371,7 +13371,7 @@
         <v>10</v>
       </c>
       <c r="F491">
-        <v>498</v>
+        <v>729</v>
       </c>
     </row>
     <row r="492" spans="1:6" x14ac:dyDescent="0.25">
@@ -13391,7 +13391,7 @@
         <v>10</v>
       </c>
       <c r="F492">
-        <v>469</v>
+        <v>546</v>
       </c>
     </row>
     <row r="493" spans="1:6" x14ac:dyDescent="0.25">
@@ -13411,7 +13411,7 @@
         <v>10</v>
       </c>
       <c r="F493">
-        <v>962</v>
+        <v>737</v>
       </c>
     </row>
     <row r="494" spans="1:6" x14ac:dyDescent="0.25">
@@ -13431,7 +13431,7 @@
         <v>10</v>
       </c>
       <c r="F494">
-        <v>291</v>
+        <v>306</v>
       </c>
     </row>
     <row r="495" spans="1:6" x14ac:dyDescent="0.25">
@@ -13451,7 +13451,7 @@
         <v>10</v>
       </c>
       <c r="F495">
-        <v>404</v>
+        <v>817</v>
       </c>
     </row>
     <row r="496" spans="1:6" x14ac:dyDescent="0.25">
@@ -13471,7 +13471,7 @@
         <v>10</v>
       </c>
       <c r="F496">
-        <v>874</v>
+        <v>245</v>
       </c>
     </row>
     <row r="497" spans="1:6" x14ac:dyDescent="0.25">
@@ -13491,7 +13491,7 @@
         <v>10</v>
       </c>
       <c r="F497">
-        <v>730</v>
+        <v>339</v>
       </c>
     </row>
     <row r="498" spans="1:6" x14ac:dyDescent="0.25">
@@ -13511,7 +13511,7 @@
         <v>10</v>
       </c>
       <c r="F498">
-        <v>539</v>
+        <v>580</v>
       </c>
     </row>
     <row r="499" spans="1:6" x14ac:dyDescent="0.25">
@@ -13531,7 +13531,7 @@
         <v>10</v>
       </c>
       <c r="F499">
-        <v>791</v>
+        <v>764</v>
       </c>
     </row>
     <row r="500" spans="1:6" x14ac:dyDescent="0.25">
@@ -13551,7 +13551,7 @@
         <v>10</v>
       </c>
       <c r="F500">
-        <v>424</v>
+        <v>460</v>
       </c>
     </row>
     <row r="501" spans="1:6" x14ac:dyDescent="0.25">
@@ -13571,7 +13571,7 @@
         <v>10</v>
       </c>
       <c r="F501">
-        <v>238</v>
+        <v>538</v>
       </c>
     </row>
     <row r="502" spans="1:6" x14ac:dyDescent="0.25">
@@ -13591,7 +13591,7 @@
         <v>10</v>
       </c>
       <c r="F502">
-        <v>955</v>
+        <v>505</v>
       </c>
     </row>
     <row r="503" spans="1:6" x14ac:dyDescent="0.25">
@@ -13611,7 +13611,7 @@
         <v>10</v>
       </c>
       <c r="F503">
-        <v>237</v>
+        <v>210</v>
       </c>
     </row>
     <row r="504" spans="1:6" x14ac:dyDescent="0.25">
@@ -13631,7 +13631,7 @@
         <v>10</v>
       </c>
       <c r="F504">
-        <v>911</v>
+        <v>822</v>
       </c>
     </row>
     <row r="505" spans="1:6" x14ac:dyDescent="0.25">
@@ -13651,7 +13651,7 @@
         <v>10</v>
       </c>
       <c r="F505">
-        <v>334</v>
+        <v>316</v>
       </c>
     </row>
     <row r="506" spans="1:6" x14ac:dyDescent="0.25">
@@ -13671,7 +13671,7 @@
         <v>10</v>
       </c>
       <c r="F506">
-        <v>545</v>
+        <v>620</v>
       </c>
     </row>
     <row r="507" spans="1:6" x14ac:dyDescent="0.25">
@@ -13691,7 +13691,7 @@
         <v>10</v>
       </c>
       <c r="F507">
-        <v>648</v>
+        <v>317</v>
       </c>
     </row>
     <row r="508" spans="1:6" x14ac:dyDescent="0.25">
@@ -13711,7 +13711,7 @@
         <v>10</v>
       </c>
       <c r="F508">
-        <v>219</v>
+        <v>418</v>
       </c>
     </row>
     <row r="509" spans="1:6" x14ac:dyDescent="0.25">
@@ -13731,7 +13731,7 @@
         <v>10</v>
       </c>
       <c r="F509">
-        <v>710</v>
+        <v>507</v>
       </c>
     </row>
     <row r="510" spans="1:6" x14ac:dyDescent="0.25">
@@ -13751,7 +13751,7 @@
         <v>10</v>
       </c>
       <c r="F510">
-        <v>365</v>
+        <v>457</v>
       </c>
     </row>
     <row r="511" spans="1:6" x14ac:dyDescent="0.25">
@@ -13771,7 +13771,7 @@
         <v>10</v>
       </c>
       <c r="F511">
-        <v>813</v>
+        <v>338</v>
       </c>
     </row>
   </sheetData>

</xml_diff>